<commit_message>
Save latest country-source and tax reporting updates
</commit_message>
<xml_diff>
--- a/docs/phase-8/export-evidence/synthetic-localfile.xlsx
+++ b/docs/phase-8/export-evidence/synthetic-localfile.xlsx
@@ -483,7 +483,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>ecfbb0fa-ebfc-407e-89ba-d1ce4da270fd / auditos-tp/1.0</t>
+          <t>342f126e-d16f-4cac-bec8-2c13a4833ba3 / auditos-tp/1.0</t>
         </is>
       </c>
     </row>
@@ -507,7 +507,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>9f2c27d589631f58d622b46242fc35a386dc3437e0fd152c7bed3f9a88d7ea03</t>
+          <t>099843472321e21f9215341804f6d400dbc19e6b8e845127925240acdd6fbd05</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>383073ea-6483-447a-8c74-fb38b6226a58</t>
+          <t>26e3325b-a5cb-418e-8025-167c64388709</t>
         </is>
       </c>
     </row>
@@ -605,7 +605,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>383073ea-6483-447a-8c74-fb38b6226a58</t>
+          <t>26e3325b-a5cb-418e-8025-167c64388709</t>
         </is>
       </c>
     </row>
@@ -636,7 +636,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>383073ea-6483-447a-8c74-fb38b6226a58</t>
+          <t>26e3325b-a5cb-418e-8025-167c64388709</t>
         </is>
       </c>
     </row>
@@ -667,7 +667,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>383073ea-6483-447a-8c74-fb38b6226a58</t>
+          <t>26e3325b-a5cb-418e-8025-167c64388709</t>
         </is>
       </c>
     </row>
@@ -698,7 +698,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>383073ea-6483-447a-8c74-fb38b6226a58</t>
+          <t>26e3325b-a5cb-418e-8025-167c64388709</t>
         </is>
       </c>
     </row>
@@ -729,7 +729,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>383073ea-6483-447a-8c74-fb38b6226a58</t>
+          <t>26e3325b-a5cb-418e-8025-167c64388709</t>
         </is>
       </c>
     </row>
@@ -741,7 +741,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>9f1251fa-b233-4ecd-9d23-99b681941173</t>
+          <t>4728be13-cd4e-4cff-b944-aaa72314e339</t>
         </is>
       </c>
     </row>
@@ -772,7 +772,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>383073ea-6483-447a-8c74-fb38b6226a58</t>
+          <t>26e3325b-a5cb-418e-8025-167c64388709</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>fdb9fdcd-b9c1-4573-a126-230767690bb4</t>
+          <t>e94f2c1e-966f-4abb-87a5-66d8467d8f35</t>
         </is>
       </c>
     </row>
@@ -834,7 +834,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>caded7dc-f14d-4d3e-9103-8ceb4c8dd3ac</t>
+          <t>98678ad6-7d06-424d-ac6a-0c1f973f72ed</t>
         </is>
       </c>
     </row>
@@ -865,7 +865,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>383073ea-6483-447a-8c74-fb38b6226a58</t>
+          <t>26e3325b-a5cb-418e-8025-167c64388709</t>
         </is>
       </c>
     </row>
@@ -896,7 +896,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>383073ea-6483-447a-8c74-fb38b6226a58</t>
+          <t>26e3325b-a5cb-418e-8025-167c64388709</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>59896288-0bc4-4ef3-9045-b5dfac9177de</t>
+          <t>8a856c62-8985-46d5-913a-50057385d3f4</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>383073ea-6483-447a-8c74-fb38b6226a58</t>
+          <t>26e3325b-a5cb-418e-8025-167c64388709</t>
         </is>
       </c>
     </row>
@@ -970,7 +970,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>383073ea-6483-447a-8c74-fb38b6226a58</t>
+          <t>26e3325b-a5cb-418e-8025-167c64388709</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>383073ea-6483-447a-8c74-fb38b6226a58</t>
+          <t>26e3325b-a5cb-418e-8025-167c64388709</t>
         </is>
       </c>
     </row>
@@ -1013,7 +1013,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>9f1251fa-b233-4ecd-9d23-99b681941173</t>
+          <t>4728be13-cd4e-4cff-b944-aaa72314e339</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1049,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>59896288-0bc4-4ef3-9045-b5dfac9177de</t>
+          <t>8a856c62-8985-46d5-913a-50057385d3f4</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "fba122e6-a861-4885-a671-2af0427f0fb7",</t>
+          <t xml:space="preserve">    "id": "5d6b30ea-667e-4f01-8d3b-219507024f74",</t>
         </is>
       </c>
     </row>
@@ -1266,7 +1266,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "8fe5bdc8-1093-4d49-8f15-90410db4e1e3",</t>
+          <t xml:space="preserve">    "id": "5151ae5a-ab3c-4239-9116-57444f6179d2",</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1301,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "dbf3317a-59a9-402c-ba5b-10b1b400241c",</t>
+          <t xml:space="preserve">    "id": "07be194f-aefb-4021-891f-f42b00d1d380",</t>
         </is>
       </c>
     </row>
@@ -1336,7 +1336,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "383073ea-6483-447a-8c74-fb38b6226a58",</t>
+          <t xml:space="preserve">    "id": "26e3325b-a5cb-418e-8025-167c64388709",</t>
         </is>
       </c>
     </row>
@@ -1371,7 +1371,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "59ca1c3b-9f10-4420-a563-de85bfd450e3",</t>
+          <t xml:space="preserve">    "id": "8111fdc0-a0c3-4220-8d4f-506d02e02aed",</t>
         </is>
       </c>
     </row>
@@ -1406,7 +1406,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "697585b8-3531-4640-925d-f04faec2c8b6",</t>
+          <t xml:space="preserve">    "id": "c5f2f746-f2ee-44cb-987c-56136d5c2de1",</t>
         </is>
       </c>
     </row>
@@ -1441,7 +1441,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "515c2499-1c25-477a-be19-599581b605ff",</t>
+          <t xml:space="preserve">    "id": "b7bc0e8e-c44c-4000-bc9b-6575a6a3f090",</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1476,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "cc5edb4c-b679-4bfb-8f5c-92c60a7455fb",</t>
+          <t xml:space="preserve">    "id": "bec5f73f-4547-4fa6-b494-4636bbb1ae62",</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1511,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "75f25a9d-d846-445a-84a3-47cfd15c89ca",</t>
+          <t xml:space="preserve">    "id": "3bcba9a4-298d-403c-bd92-b88dcd0de1e6",</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "092d6bde-2841-4ef9-9d18-c01e78611952",</t>
+          <t xml:space="preserve">    "id": "eaf1cd80-da44-4287-9129-98e9e720b8a0",</t>
         </is>
       </c>
     </row>
@@ -1581,7 +1581,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "979752dc-31f7-417a-8724-59dc251c823f",</t>
+          <t xml:space="preserve">    "id": "6a96a1eb-21dd-4cd6-b52d-39e1d24c5c8b",</t>
         </is>
       </c>
     </row>
@@ -1616,7 +1616,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "6e9a8d48-f8fd-4609-b907-cfed7ebb2312",</t>
+          <t xml:space="preserve">    "id": "0a129ba1-1e8f-490f-8b33-748d6c2db1f3",</t>
         </is>
       </c>
     </row>
@@ -1665,7 +1665,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "414fe600-3da4-49aa-818e-682e7ff12ee9",</t>
+          <t xml:space="preserve">    "id": "f387e7fd-fe7a-4fff-893c-f1eb47aa0ed3",</t>
         </is>
       </c>
     </row>
@@ -1714,7 +1714,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "e5e6af42-61a4-4860-8d74-366cdf0e170c",</t>
+          <t xml:space="preserve">    "id": "33ed8bae-2f18-4b6a-8347-39373f58e484",</t>
         </is>
       </c>
     </row>
@@ -1763,7 +1763,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "46495fd8-4d00-44a0-be16-adc6dbbb38c9",</t>
+          <t xml:space="preserve">    "id": "63b9bd2c-df96-469f-82d3-857205b0f694",</t>
         </is>
       </c>
     </row>
@@ -1812,7 +1812,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "54f18b07-b4cf-4405-9fe2-fd35d1245db7",</t>
+          <t xml:space="preserve">    "id": "134ca4a1-d675-4d20-a5cc-25061178240b",</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "634078e1-cba6-4e97-b213-f6b5d5c0c729",</t>
+          <t xml:space="preserve">    "id": "749bfec7-47a7-4cfb-919f-6c420f9fc15f",</t>
         </is>
       </c>
     </row>
@@ -1910,7 +1910,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "30f134e4-9320-4637-86c8-c08b0b422abb",</t>
+          <t xml:space="preserve">    "id": "a4399843-db68-4b86-8733-f33e5245e9c0",</t>
         </is>
       </c>
     </row>
@@ -1959,7 +1959,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "acc88b17-2731-439a-9376-1efb4a18ff87",</t>
+          <t xml:space="preserve">    "id": "599f6bca-5333-467c-bbc9-5b60b04c9b3e",</t>
         </is>
       </c>
     </row>
@@ -2008,7 +2008,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "59b42a56-53d1-4e78-ac48-7b302efed0c2",</t>
+          <t xml:space="preserve">    "id": "d56ca2f7-3b45-4fc5-87b1-a298cb1f4645",</t>
         </is>
       </c>
     </row>
@@ -2057,14 +2057,14 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "caded7dc-f14d-4d3e-9103-8ceb4c8dd3ac",</t>
+          <t xml:space="preserve">    "id": "26e3325b-a5cb-418e-8025-167c64388709",</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "kind": "tp-method",</t>
+          <t xml:space="preserve">    "kind": "ifrs-note",</t>
         </is>
       </c>
     </row>
@@ -2106,14 +2106,14 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "fdb9fdcd-b9c1-4573-a126-230767690bb4",</t>
+          <t xml:space="preserve">    "id": "98678ad6-7d06-424d-ac6a-0c1f973f72ed",</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "kind": "tp-far",</t>
+          <t xml:space="preserve">    "kind": "tp-method",</t>
         </is>
       </c>
     </row>
@@ -2155,14 +2155,14 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "383073ea-6483-447a-8c74-fb38b6226a58",</t>
+          <t xml:space="preserve">    "id": "e94f2c1e-966f-4abb-87a5-66d8467d8f35",</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "kind": "ifrs-note",</t>
+          <t xml:space="preserve">    "kind": "tp-far",</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2204,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "64db4a8a-54e5-40a7-8654-4a16cd084ed7",</t>
+          <t xml:space="preserve">    "id": "ad4c54ff-da6c-4474-a0d7-99c82e42ba9b",</t>
         </is>
       </c>
     </row>
@@ -2253,7 +2253,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "8d3d9472-dd0e-4e55-ac64-2e8c2cecbfc9",</t>
+          <t xml:space="preserve">    "id": "249b5cc3-1aa2-4fc2-a638-fa4a21f8b192",</t>
         </is>
       </c>
     </row>
@@ -2302,7 +2302,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "7c6f52dd-0b10-4849-bb5b-63937e8b3f7a",</t>
+          <t xml:space="preserve">    "id": "0ceeb1f1-b2a2-43ec-8d87-840f74b2dd70",</t>
         </is>
       </c>
     </row>
@@ -2351,7 +2351,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "26997a51-b558-43e8-a18b-8bcb0385cfe6",</t>
+          <t xml:space="preserve">    "id": "60346b5b-473b-4889-a5da-68b017ca186b",</t>
         </is>
       </c>
     </row>
@@ -2400,7 +2400,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "5fdd6fbd-f1f1-4e9c-80b8-f76c0a7d4293",</t>
+          <t xml:space="preserve">    "id": "8534d3b8-8b3a-44de-b207-57cc951802f9",</t>
         </is>
       </c>
     </row>
@@ -2449,7 +2449,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "634078e1-cba6-4e97-b213-f6b5d5c0c729",</t>
+          <t xml:space="preserve">    "id": "749bfec7-47a7-4cfb-919f-6c420f9fc15f",</t>
         </is>
       </c>
     </row>
@@ -2498,7 +2498,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "9f1251fa-b233-4ecd-9d23-99b681941173",</t>
+          <t xml:space="preserve">    "id": "4728be13-cd4e-4cff-b944-aaa72314e339",</t>
         </is>
       </c>
     </row>
@@ -2512,7 +2512,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "sha256": "4abe92101801f412f14c63a55305380d3ce93db85011148e89d4401f451873aa"</t>
+          <t xml:space="preserve">    "sha256": "bb6f6c59ca6fe7f3b2a629ba29c663b12a97df4414d9aad8e355a7a861a82292"</t>
         </is>
       </c>
     </row>
@@ -2533,7 +2533,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "5361f161-7a01-4173-a92e-a24f2285d076",</t>
+          <t xml:space="preserve">    "id": "3ad8dcc4-73bb-4757-860b-d47162b2a4cf",</t>
         </is>
       </c>
     </row>
@@ -2547,7 +2547,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "sha256": "06691a9635e7694772fa02a48b97c4543778bd2c484c0845dab710f92384f4a5"</t>
+          <t xml:space="preserve">    "sha256": "938fe13b721d15eebe42e4915709301cad961dd4f53e781a1f34575768e4a668"</t>
         </is>
       </c>
     </row>
@@ -2568,7 +2568,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "59896288-0bc4-4ef3-9045-b5dfac9177de",</t>
+          <t xml:space="preserve">    "id": "8a856c62-8985-46d5-913a-50057385d3f4",</t>
         </is>
       </c>
     </row>
@@ -2582,7 +2582,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "sha256": "09fbdfee5c061267875b5ed8b9767c4068a3c86a466e2f7464e3e39c653017a6"</t>
+          <t xml:space="preserve">    "sha256": "11a5e9130b9b012d21bd7ed155d7173f79fb0221274b4c0d06f2ac557133d3bf"</t>
         </is>
       </c>
     </row>
@@ -2611,7 +2611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1376"/>
+  <dimension ref="A1:A1381"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -2627,14 +2627,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  "id": "ecfbb0fa-ebfc-407e-89ba-d1ce4da270fd",</t>
+          <t xml:space="preserve">  "id": "342f126e-d16f-4cac-bec8-2c13a4833ba3",</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  "sha256": "9f2c27d589631f58d622b46242fc35a386dc3437e0fd152c7bed3f9a88d7ea03",</t>
+          <t xml:space="preserve">  "sha256": "099843472321e21f9215341804f6d400dbc19e6b8e845127925240acdd6fbd05",</t>
         </is>
       </c>
     </row>
@@ -2655,14 +2655,14 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  "prepared_by": "fc84e85f-5daf-4922-94ec-3769b3209b34",</t>
+          <t xml:space="preserve">  "prepared_by": "368c7cfa-ac0d-4a06-a71c-247c923c7eee",</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  "created_at": "2026-10-24 18:15:34.799967+00:00",</t>
+          <t xml:space="preserve">  "created_at": "2026-10-24 18:34:29.653566+00:00",</t>
         </is>
       </c>
     </row>
@@ -2683,14 +2683,14 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "record_id": "59b42a56-53d1-4e78-ac48-7b302efed0c2",</t>
+          <t xml:space="preserve">    "record_id": "d56ca2f7-3b45-4fc5-87b1-a298cb1f4645",</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "profile_id": "6e9a8d48-f8fd-4609-b907-cfed7ebb2312"</t>
+          <t xml:space="preserve">    "profile_id": "0a129ba1-1e8f-490f-8b33-748d6c2db1f3"</t>
         </is>
       </c>
     </row>
@@ -2718,7 +2718,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "fba122e6-a861-4885-a671-2af0427f0fb7",</t>
+          <t xml:space="preserve">      "id": "5d6b30ea-667e-4f01-8d3b-219507024f74",</t>
         </is>
       </c>
     </row>
@@ -2753,7 +2753,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "8fe5bdc8-1093-4d49-8f15-90410db4e1e3",</t>
+          <t xml:space="preserve">      "id": "5151ae5a-ab3c-4239-9116-57444f6179d2",</t>
         </is>
       </c>
     </row>
@@ -2788,7 +2788,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "dbf3317a-59a9-402c-ba5b-10b1b400241c",</t>
+          <t xml:space="preserve">      "id": "07be194f-aefb-4021-891f-f42b00d1d380",</t>
         </is>
       </c>
     </row>
@@ -2823,7 +2823,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "383073ea-6483-447a-8c74-fb38b6226a58",</t>
+          <t xml:space="preserve">      "id": "26e3325b-a5cb-418e-8025-167c64388709",</t>
         </is>
       </c>
     </row>
@@ -2858,7 +2858,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "59ca1c3b-9f10-4420-a563-de85bfd450e3",</t>
+          <t xml:space="preserve">      "id": "8111fdc0-a0c3-4220-8d4f-506d02e02aed",</t>
         </is>
       </c>
     </row>
@@ -2893,7 +2893,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "697585b8-3531-4640-925d-f04faec2c8b6",</t>
+          <t xml:space="preserve">      "id": "c5f2f746-f2ee-44cb-987c-56136d5c2de1",</t>
         </is>
       </c>
     </row>
@@ -2928,7 +2928,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "515c2499-1c25-477a-be19-599581b605ff",</t>
+          <t xml:space="preserve">      "id": "b7bc0e8e-c44c-4000-bc9b-6575a6a3f090",</t>
         </is>
       </c>
     </row>
@@ -2963,7 +2963,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "cc5edb4c-b679-4bfb-8f5c-92c60a7455fb",</t>
+          <t xml:space="preserve">      "id": "bec5f73f-4547-4fa6-b494-4636bbb1ae62",</t>
         </is>
       </c>
     </row>
@@ -2998,7 +2998,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "75f25a9d-d846-445a-84a3-47cfd15c89ca",</t>
+          <t xml:space="preserve">      "id": "3bcba9a4-298d-403c-bd92-b88dcd0de1e6",</t>
         </is>
       </c>
     </row>
@@ -3033,7 +3033,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "092d6bde-2841-4ef9-9d18-c01e78611952",</t>
+          <t xml:space="preserve">      "id": "eaf1cd80-da44-4287-9129-98e9e720b8a0",</t>
         </is>
       </c>
     </row>
@@ -3068,7 +3068,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "979752dc-31f7-417a-8724-59dc251c823f",</t>
+          <t xml:space="preserve">      "id": "6a96a1eb-21dd-4cd6-b52d-39e1d24c5c8b",</t>
         </is>
       </c>
     </row>
@@ -3103,7 +3103,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "6e9a8d48-f8fd-4609-b907-cfed7ebb2312",</t>
+          <t xml:space="preserve">      "id": "0a129ba1-1e8f-490f-8b33-748d6c2db1f3",</t>
         </is>
       </c>
     </row>
@@ -3152,7 +3152,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "414fe600-3da4-49aa-818e-682e7ff12ee9",</t>
+          <t xml:space="preserve">      "id": "f387e7fd-fe7a-4fff-893c-f1eb47aa0ed3",</t>
         </is>
       </c>
     </row>
@@ -3201,7 +3201,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "e5e6af42-61a4-4860-8d74-366cdf0e170c",</t>
+          <t xml:space="preserve">      "id": "33ed8bae-2f18-4b6a-8347-39373f58e484",</t>
         </is>
       </c>
     </row>
@@ -3250,7 +3250,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "46495fd8-4d00-44a0-be16-adc6dbbb38c9",</t>
+          <t xml:space="preserve">      "id": "63b9bd2c-df96-469f-82d3-857205b0f694",</t>
         </is>
       </c>
     </row>
@@ -3299,7 +3299,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "54f18b07-b4cf-4405-9fe2-fd35d1245db7",</t>
+          <t xml:space="preserve">      "id": "134ca4a1-d675-4d20-a5cc-25061178240b",</t>
         </is>
       </c>
     </row>
@@ -3348,7 +3348,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "634078e1-cba6-4e97-b213-f6b5d5c0c729",</t>
+          <t xml:space="preserve">      "id": "749bfec7-47a7-4cfb-919f-6c420f9fc15f",</t>
         </is>
       </c>
     </row>
@@ -3397,7 +3397,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "30f134e4-9320-4637-86c8-c08b0b422abb",</t>
+          <t xml:space="preserve">      "id": "a4399843-db68-4b86-8733-f33e5245e9c0",</t>
         </is>
       </c>
     </row>
@@ -3446,7 +3446,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "acc88b17-2731-439a-9376-1efb4a18ff87",</t>
+          <t xml:space="preserve">      "id": "599f6bca-5333-467c-bbc9-5b60b04c9b3e",</t>
         </is>
       </c>
     </row>
@@ -3495,7 +3495,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "59b42a56-53d1-4e78-ac48-7b302efed0c2",</t>
+          <t xml:space="preserve">      "id": "d56ca2f7-3b45-4fc5-87b1-a298cb1f4645",</t>
         </is>
       </c>
     </row>
@@ -3544,14 +3544,14 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "caded7dc-f14d-4d3e-9103-8ceb4c8dd3ac",</t>
+          <t xml:space="preserve">      "id": "26e3325b-a5cb-418e-8025-167c64388709",</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "kind": "tp-method",</t>
+          <t xml:space="preserve">      "kind": "ifrs-note",</t>
         </is>
       </c>
     </row>
@@ -3593,14 +3593,14 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "fdb9fdcd-b9c1-4573-a126-230767690bb4",</t>
+          <t xml:space="preserve">      "id": "98678ad6-7d06-424d-ac6a-0c1f973f72ed",</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "kind": "tp-far",</t>
+          <t xml:space="preserve">      "kind": "tp-method",</t>
         </is>
       </c>
     </row>
@@ -3642,14 +3642,14 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "383073ea-6483-447a-8c74-fb38b6226a58",</t>
+          <t xml:space="preserve">      "id": "e94f2c1e-966f-4abb-87a5-66d8467d8f35",</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "kind": "ifrs-note",</t>
+          <t xml:space="preserve">      "kind": "tp-far",</t>
         </is>
       </c>
     </row>
@@ -3691,7 +3691,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "64db4a8a-54e5-40a7-8654-4a16cd084ed7",</t>
+          <t xml:space="preserve">      "id": "ad4c54ff-da6c-4474-a0d7-99c82e42ba9b",</t>
         </is>
       </c>
     </row>
@@ -3740,7 +3740,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "8d3d9472-dd0e-4e55-ac64-2e8c2cecbfc9",</t>
+          <t xml:space="preserve">      "id": "249b5cc3-1aa2-4fc2-a638-fa4a21f8b192",</t>
         </is>
       </c>
     </row>
@@ -3789,7 +3789,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "7c6f52dd-0b10-4849-bb5b-63937e8b3f7a",</t>
+          <t xml:space="preserve">      "id": "0ceeb1f1-b2a2-43ec-8d87-840f74b2dd70",</t>
         </is>
       </c>
     </row>
@@ -3838,7 +3838,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "26997a51-b558-43e8-a18b-8bcb0385cfe6",</t>
+          <t xml:space="preserve">      "id": "60346b5b-473b-4889-a5da-68b017ca186b",</t>
         </is>
       </c>
     </row>
@@ -3887,7 +3887,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "5fdd6fbd-f1f1-4e9c-80b8-f76c0a7d4293",</t>
+          <t xml:space="preserve">      "id": "8534d3b8-8b3a-44de-b207-57cc951802f9",</t>
         </is>
       </c>
     </row>
@@ -3936,7 +3936,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "634078e1-cba6-4e97-b213-f6b5d5c0c729",</t>
+          <t xml:space="preserve">      "id": "749bfec7-47a7-4cfb-919f-6c420f9fc15f",</t>
         </is>
       </c>
     </row>
@@ -3985,7 +3985,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "9f1251fa-b233-4ecd-9d23-99b681941173",</t>
+          <t xml:space="preserve">      "id": "4728be13-cd4e-4cff-b944-aaa72314e339",</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "sha256": "4abe92101801f412f14c63a55305380d3ce93db85011148e89d4401f451873aa"</t>
+          <t xml:space="preserve">      "sha256": "bb6f6c59ca6fe7f3b2a629ba29c663b12a97df4414d9aad8e355a7a861a82292"</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "5361f161-7a01-4173-a92e-a24f2285d076",</t>
+          <t xml:space="preserve">      "id": "3ad8dcc4-73bb-4757-860b-d47162b2a4cf",</t>
         </is>
       </c>
     </row>
@@ -4034,7 +4034,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "sha256": "06691a9635e7694772fa02a48b97c4543778bd2c484c0845dab710f92384f4a5"</t>
+          <t xml:space="preserve">      "sha256": "938fe13b721d15eebe42e4915709301cad961dd4f53e781a1f34575768e4a668"</t>
         </is>
       </c>
     </row>
@@ -4055,7 +4055,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "59896288-0bc4-4ef3-9045-b5dfac9177de",</t>
+          <t xml:space="preserve">      "id": "8a856c62-8985-46d5-913a-50057385d3f4",</t>
         </is>
       </c>
     </row>
@@ -4069,7 +4069,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "sha256": "09fbdfee5c061267875b5ed8b9767c4068a3c86a466e2f7464e3e39c653017a6"</t>
+          <t xml:space="preserve">      "sha256": "11a5e9130b9b012d21bd7ed155d7173f79fb0221274b4c0d06f2ac557133d3bf"</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t xml:space="preserve">            "e46262e7-fad4-498f-a048-cbdce542c22a"</t>
+          <t xml:space="preserve">            "da75be6b-463d-44e4-8dc4-1e26094a7ff7"</t>
         </is>
       </c>
     </row>
@@ -4349,7 +4349,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "rule_record_id": "414fe600-3da4-49aa-818e-682e7ff12ee9",</t>
+          <t xml:space="preserve">        "rule_record_id": "f387e7fd-fe7a-4fff-893c-f1eb47aa0ed3",</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t xml:space="preserve">            "e46262e7-fad4-498f-a048-cbdce542c22a"</t>
+          <t xml:space="preserve">            "da75be6b-463d-44e4-8dc4-1e26094a7ff7"</t>
         </is>
       </c>
     </row>
@@ -4706,7 +4706,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "rule_record_id": "e5e6af42-61a4-4860-8d74-366cdf0e170c",</t>
+          <t xml:space="preserve">        "rule_record_id": "33ed8bae-2f18-4b6a-8347-39373f58e484",</t>
         </is>
       </c>
     </row>
@@ -5014,7 +5014,7 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t xml:space="preserve">            "e46262e7-fad4-498f-a048-cbdce542c22a"</t>
+          <t xml:space="preserve">            "da75be6b-463d-44e4-8dc4-1e26094a7ff7"</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "rule_record_id": "46495fd8-4d00-44a0-be16-adc6dbbb38c9",</t>
+          <t xml:space="preserve">        "rule_record_id": "63b9bd2c-df96-469f-82d3-857205b0f694",</t>
         </is>
       </c>
     </row>
@@ -5399,7 +5399,7 @@
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t xml:space="preserve">            "e46262e7-fad4-498f-a048-cbdce542c22a"</t>
+          <t xml:space="preserve">            "da75be6b-463d-44e4-8dc4-1e26094a7ff7"</t>
         </is>
       </c>
     </row>
@@ -5434,7 +5434,7 @@
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "rule_record_id": "54f18b07-b4cf-4405-9fe2-fd35d1245db7",</t>
+          <t xml:space="preserve">        "rule_record_id": "134ca4a1-d675-4d20-a5cc-25061178240b",</t>
         </is>
       </c>
     </row>
@@ -5749,7 +5749,7 @@
     <row r="448">
       <c r="A448" t="inlineStr">
         <is>
-          <t xml:space="preserve">            "e46262e7-fad4-498f-a048-cbdce542c22a"</t>
+          <t xml:space="preserve">            "da75be6b-463d-44e4-8dc4-1e26094a7ff7"</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "rule_record_id": "634078e1-cba6-4e97-b213-f6b5d5c0c729",</t>
+          <t xml:space="preserve">        "rule_record_id": "749bfec7-47a7-4cfb-919f-6c420f9fc15f",</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
     <row r="498">
       <c r="A498" t="inlineStr">
         <is>
-          <t xml:space="preserve">            "e46262e7-fad4-498f-a048-cbdce542c22a"</t>
+          <t xml:space="preserve">            "da75be6b-463d-44e4-8dc4-1e26094a7ff7"</t>
         </is>
       </c>
     </row>
@@ -6134,7 +6134,7 @@
     <row r="503">
       <c r="A503" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "rule_record_id": "30f134e4-9320-4637-86c8-c08b0b422abb",</t>
+          <t xml:space="preserve">        "rule_record_id": "a4399843-db68-4b86-8733-f33e5245e9c0",</t>
         </is>
       </c>
     </row>
@@ -6449,7 +6449,7 @@
     <row r="548">
       <c r="A548" t="inlineStr">
         <is>
-          <t xml:space="preserve">            "e46262e7-fad4-498f-a048-cbdce542c22a"</t>
+          <t xml:space="preserve">            "da75be6b-463d-44e4-8dc4-1e26094a7ff7"</t>
         </is>
       </c>
     </row>
@@ -6484,7 +6484,7 @@
     <row r="553">
       <c r="A553" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "rule_record_id": "acc88b17-2731-439a-9376-1efb4a18ff87",</t>
+          <t xml:space="preserve">        "rule_record_id": "599f6bca-5333-467c-bbc9-5b60b04c9b3e",</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
     <row r="576">
       <c r="A576" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "383073ea-6483-447a-8c74-fb38b6226a58"</t>
+          <t xml:space="preserve">          "26e3325b-a5cb-418e-8025-167c64388709"</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
     <row r="585">
       <c r="A585" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "383073ea-6483-447a-8c74-fb38b6226a58"</t>
+          <t xml:space="preserve">          "26e3325b-a5cb-418e-8025-167c64388709"</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
     <row r="594">
       <c r="A594" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "383073ea-6483-447a-8c74-fb38b6226a58"</t>
+          <t xml:space="preserve">          "26e3325b-a5cb-418e-8025-167c64388709"</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
     <row r="603">
       <c r="A603" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "383073ea-6483-447a-8c74-fb38b6226a58"</t>
+          <t xml:space="preserve">          "26e3325b-a5cb-418e-8025-167c64388709"</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
     <row r="612">
       <c r="A612" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "383073ea-6483-447a-8c74-fb38b6226a58"</t>
+          <t xml:space="preserve">          "26e3325b-a5cb-418e-8025-167c64388709"</t>
         </is>
       </c>
     </row>
@@ -6946,7 +6946,7 @@
     <row r="619">
       <c r="A619" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "9f1251fa-b233-4ecd-9d23-99b681941173"</t>
+          <t xml:space="preserve">          "4728be13-cd4e-4cff-b944-aaa72314e339"</t>
         </is>
       </c>
     </row>
@@ -6974,7 +6974,7 @@
     <row r="623">
       <c r="A623" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "383073ea-6483-447a-8c74-fb38b6226a58"</t>
+          <t xml:space="preserve">          "26e3325b-a5cb-418e-8025-167c64388709"</t>
         </is>
       </c>
     </row>
@@ -7037,7 +7037,7 @@
     <row r="632">
       <c r="A632" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "383073ea-6483-447a-8c74-fb38b6226a58"</t>
+          <t xml:space="preserve">          "26e3325b-a5cb-418e-8025-167c64388709"</t>
         </is>
       </c>
     </row>
@@ -7100,7 +7100,7 @@
     <row r="641">
       <c r="A641" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "fdb9fdcd-b9c1-4573-a126-230767690bb4"</t>
+          <t xml:space="preserve">          "e94f2c1e-966f-4abb-87a5-66d8467d8f35"</t>
         </is>
       </c>
     </row>
@@ -7163,7 +7163,7 @@
     <row r="650">
       <c r="A650" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "caded7dc-f14d-4d3e-9103-8ceb4c8dd3ac"</t>
+          <t xml:space="preserve">          "98678ad6-7d06-424d-ac6a-0c1f973f72ed"</t>
         </is>
       </c>
     </row>
@@ -7226,7 +7226,7 @@
     <row r="659">
       <c r="A659" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "383073ea-6483-447a-8c74-fb38b6226a58"</t>
+          <t xml:space="preserve">          "26e3325b-a5cb-418e-8025-167c64388709"</t>
         </is>
       </c>
     </row>
@@ -7275,7 +7275,7 @@
     <row r="666">
       <c r="A666" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "59896288-0bc4-4ef3-9045-b5dfac9177de"</t>
+          <t xml:space="preserve">          "8a856c62-8985-46d5-913a-50057385d3f4"</t>
         </is>
       </c>
     </row>
@@ -7303,7 +7303,7 @@
     <row r="670">
       <c r="A670" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "383073ea-6483-447a-8c74-fb38b6226a58"</t>
+          <t xml:space="preserve">          "26e3325b-a5cb-418e-8025-167c64388709"</t>
         </is>
       </c>
     </row>
@@ -7366,7 +7366,7 @@
     <row r="679">
       <c r="A679" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "383073ea-6483-447a-8c74-fb38b6226a58"</t>
+          <t xml:space="preserve">          "26e3325b-a5cb-418e-8025-167c64388709"</t>
         </is>
       </c>
     </row>
@@ -7429,7 +7429,7 @@
     <row r="688">
       <c r="A688" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "383073ea-6483-447a-8c74-fb38b6226a58"</t>
+          <t xml:space="preserve">          "26e3325b-a5cb-418e-8025-167c64388709"</t>
         </is>
       </c>
     </row>
@@ -7492,7 +7492,7 @@
     <row r="697">
       <c r="A697" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "383073ea-6483-447a-8c74-fb38b6226a58"</t>
+          <t xml:space="preserve">          "26e3325b-a5cb-418e-8025-167c64388709"</t>
         </is>
       </c>
     </row>
@@ -7527,7 +7527,7 @@
     <row r="702">
       <c r="A702" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "entity_id": "00818376-5b2e-4cac-91ac-c24aa237221b",</t>
+          <t xml:space="preserve">    "entity_id": "26047f96-aba9-4e5f-97eb-a04d18c3e2ce",</t>
         </is>
       </c>
     </row>
@@ -7548,7 +7548,7 @@
     <row r="705">
       <c r="A705" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "profile_id": "6e9a8d48-f8fd-4609-b907-cfed7ebb2312",</t>
+          <t xml:space="preserve">    "profile_id": "0a129ba1-1e8f-490f-8b33-748d6c2db1f3",</t>
         </is>
       </c>
     </row>
@@ -7597,21 +7597,21 @@
     <row r="712">
       <c r="A712" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "entity_id": "00818376-5b2e-4cac-91ac-c24aa237221b",</t>
+          <t xml:space="preserve">      "entity_id": "26047f96-aba9-4e5f-97eb-a04d18c3e2ce",</t>
         </is>
       </c>
     </row>
     <row r="713">
       <c r="A713" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "period_id": "59bda27d-f8a8-4b3d-a618-87f20488ba0d",</t>
+          <t xml:space="preserve">      "period_id": "075ce9a3-fc18-4d94-b850-2f7a6e4d0e3f",</t>
         </is>
       </c>
     </row>
     <row r="714">
       <c r="A714" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "tenant_id": "af66d068-09b3-4e17-853f-7d3a21413081",</t>
+          <t xml:space="preserve">      "tenant_id": "3c52af75-856a-4d05-aed4-aa0f5f067823",</t>
         </is>
       </c>
     </row>
@@ -7646,7 +7646,7 @@
     <row r="719">
       <c r="A719" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "execution_id": "698ba3ce-bb24-43a9-9100-b576651730fa",</t>
+          <t xml:space="preserve">      "execution_id": "438cd359-30fc-4896-a3d6-f01396f930d7",</t>
         </is>
       </c>
     </row>
@@ -7660,7 +7660,7 @@
     <row r="721">
       <c r="A721" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "engagement_id": "d313758b-f840-4233-b6ca-99550d8c8043",</t>
+          <t xml:space="preserve">      "engagement_id": "8566cd98-1801-41ee-94c0-604933ca119c",</t>
         </is>
       </c>
     </row>
@@ -7891,7 +7891,7 @@
     <row r="754">
       <c r="A754" t="inlineStr">
         <is>
-          <t xml:space="preserve">              "e46262e7-fad4-498f-a048-cbdce542c22a"</t>
+          <t xml:space="preserve">              "da75be6b-463d-44e4-8dc4-1e26094a7ff7"</t>
         </is>
       </c>
     </row>
@@ -7926,7 +7926,7 @@
     <row r="759">
       <c r="A759" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "rule_record_id": "414fe600-3da4-49aa-818e-682e7ff12ee9",</t>
+          <t xml:space="preserve">          "rule_record_id": "f387e7fd-fe7a-4fff-893c-f1eb47aa0ed3",</t>
         </is>
       </c>
     </row>
@@ -8248,7 +8248,7 @@
     <row r="805">
       <c r="A805" t="inlineStr">
         <is>
-          <t xml:space="preserve">              "e46262e7-fad4-498f-a048-cbdce542c22a"</t>
+          <t xml:space="preserve">              "da75be6b-463d-44e4-8dc4-1e26094a7ff7"</t>
         </is>
       </c>
     </row>
@@ -8283,7 +8283,7 @@
     <row r="810">
       <c r="A810" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "rule_record_id": "e5e6af42-61a4-4860-8d74-366cdf0e170c",</t>
+          <t xml:space="preserve">          "rule_record_id": "33ed8bae-2f18-4b6a-8347-39373f58e484",</t>
         </is>
       </c>
     </row>
@@ -8591,7 +8591,7 @@
     <row r="854">
       <c r="A854" t="inlineStr">
         <is>
-          <t xml:space="preserve">              "e46262e7-fad4-498f-a048-cbdce542c22a"</t>
+          <t xml:space="preserve">              "da75be6b-463d-44e4-8dc4-1e26094a7ff7"</t>
         </is>
       </c>
     </row>
@@ -8626,7 +8626,7 @@
     <row r="859">
       <c r="A859" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "rule_record_id": "46495fd8-4d00-44a0-be16-adc6dbbb38c9",</t>
+          <t xml:space="preserve">          "rule_record_id": "63b9bd2c-df96-469f-82d3-857205b0f694",</t>
         </is>
       </c>
     </row>
@@ -8976,7 +8976,7 @@
     <row r="909">
       <c r="A909" t="inlineStr">
         <is>
-          <t xml:space="preserve">              "e46262e7-fad4-498f-a048-cbdce542c22a"</t>
+          <t xml:space="preserve">              "da75be6b-463d-44e4-8dc4-1e26094a7ff7"</t>
         </is>
       </c>
     </row>
@@ -9011,7 +9011,7 @@
     <row r="914">
       <c r="A914" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "rule_record_id": "54f18b07-b4cf-4405-9fe2-fd35d1245db7",</t>
+          <t xml:space="preserve">          "rule_record_id": "134ca4a1-d675-4d20-a5cc-25061178240b",</t>
         </is>
       </c>
     </row>
@@ -9326,7 +9326,7 @@
     <row r="959">
       <c r="A959" t="inlineStr">
         <is>
-          <t xml:space="preserve">              "e46262e7-fad4-498f-a048-cbdce542c22a"</t>
+          <t xml:space="preserve">              "da75be6b-463d-44e4-8dc4-1e26094a7ff7"</t>
         </is>
       </c>
     </row>
@@ -9361,7 +9361,7 @@
     <row r="964">
       <c r="A964" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "rule_record_id": "634078e1-cba6-4e97-b213-f6b5d5c0c729",</t>
+          <t xml:space="preserve">          "rule_record_id": "749bfec7-47a7-4cfb-919f-6c420f9fc15f",</t>
         </is>
       </c>
     </row>
@@ -9676,7 +9676,7 @@
     <row r="1009">
       <c r="A1009" t="inlineStr">
         <is>
-          <t xml:space="preserve">              "e46262e7-fad4-498f-a048-cbdce542c22a"</t>
+          <t xml:space="preserve">              "da75be6b-463d-44e4-8dc4-1e26094a7ff7"</t>
         </is>
       </c>
     </row>
@@ -9711,7 +9711,7 @@
     <row r="1014">
       <c r="A1014" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "rule_record_id": "30f134e4-9320-4637-86c8-c08b0b422abb",</t>
+          <t xml:space="preserve">          "rule_record_id": "a4399843-db68-4b86-8733-f33e5245e9c0",</t>
         </is>
       </c>
     </row>
@@ -10026,7 +10026,7 @@
     <row r="1059">
       <c r="A1059" t="inlineStr">
         <is>
-          <t xml:space="preserve">              "e46262e7-fad4-498f-a048-cbdce542c22a"</t>
+          <t xml:space="preserve">              "da75be6b-463d-44e4-8dc4-1e26094a7ff7"</t>
         </is>
       </c>
     </row>
@@ -10061,7 +10061,7 @@
     <row r="1064">
       <c r="A1064" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "rule_record_id": "acc88b17-2731-439a-9376-1efb4a18ff87",</t>
+          <t xml:space="preserve">          "rule_record_id": "599f6bca-5333-467c-bbc9-5b60b04c9b3e",</t>
         </is>
       </c>
     </row>
@@ -10201,2049 +10201,2084 @@
     <row r="1084">
       <c r="A1084" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "87cc43ff-587c-4ade-884f-bfc99e606f76",</t>
+          <t xml:space="preserve">          "id": "8816bb6e-d8c5-4b32-aedd-acba6f466682",</t>
         </is>
       </c>
     </row>
     <row r="1085">
       <c r="A1085" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "sha256": "6085cfbf4bfe45b540a5a50bb448d4df30ebea28df6bf25abff07a20f59be395"</t>
+          <t xml:space="preserve">          "sha256": "7ce31010c21c2309ceeee64b6f08535e9fd76e831e50de13686c36437ac5b613",</t>
         </is>
       </c>
     </row>
     <row r="1086">
       <c r="A1086" t="inlineStr">
         <is>
-          <t xml:space="preserve">        }</t>
+          <t xml:space="preserve">          "source_complete": true</t>
         </is>
       </c>
     </row>
     <row r="1087">
       <c r="A1087" t="inlineStr">
         <is>
-          <t xml:space="preserve">      ],</t>
+          <t xml:space="preserve">        }</t>
         </is>
       </c>
     </row>
     <row r="1088">
       <c r="A1088" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "accounting_amount": null,</t>
+          <t xml:space="preserve">      ],</t>
         </is>
       </c>
     </row>
     <row r="1089">
       <c r="A1089" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "input_completeness": "complete_for_supported_case",</t>
+          <t xml:space="preserve">      "accounting_amount": null,</t>
         </is>
       </c>
     </row>
     <row r="1090">
       <c r="A1090" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "calculation_version": "connected-tp/1",</t>
+          <t xml:space="preserve">      "input_completeness": "partial",</t>
         </is>
       </c>
     </row>
     <row r="1091">
       <c r="A1091" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "evidence_references": [</t>
+          <t xml:space="preserve">      "calculation_version": "connected-tp/1",</t>
         </is>
       </c>
     </row>
     <row r="1092">
       <c r="A1092" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">      "evidence_references": [</t>
         </is>
       </c>
     </row>
     <row r="1093">
       <c r="A1093" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "fba122e6-a861-4885-a671-2af0427f0fb7",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1094">
       <c r="A1094" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "id": "5d6b30ea-667e-4f01-8d3b-219507024f74",</t>
         </is>
       </c>
     </row>
     <row r="1095">
       <c r="A1095" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 3</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1096">
       <c r="A1096" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "version": 3</t>
         </is>
       </c>
     </row>
     <row r="1097">
       <c r="A1097" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1098">
       <c r="A1098" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "8fe5bdc8-1093-4d49-8f15-90410db4e1e3",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1099">
       <c r="A1099" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "id": "5151ae5a-ab3c-4239-9116-57444f6179d2",</t>
         </is>
       </c>
     </row>
     <row r="1100">
       <c r="A1100" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 3</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1101">
       <c r="A1101" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "version": 3</t>
         </is>
       </c>
     </row>
     <row r="1102">
       <c r="A1102" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1103">
       <c r="A1103" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "dbf3317a-59a9-402c-ba5b-10b1b400241c",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1104">
       <c r="A1104" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "id": "07be194f-aefb-4021-891f-f42b00d1d380",</t>
         </is>
       </c>
     </row>
     <row r="1105">
       <c r="A1105" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 3</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1106">
       <c r="A1106" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "version": 3</t>
         </is>
       </c>
     </row>
     <row r="1107">
       <c r="A1107" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1108">
       <c r="A1108" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "383073ea-6483-447a-8c74-fb38b6226a58",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1109">
       <c r="A1109" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "id": "26e3325b-a5cb-418e-8025-167c64388709",</t>
         </is>
       </c>
     </row>
     <row r="1110">
       <c r="A1110" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 3</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1111">
       <c r="A1111" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "version": 3</t>
         </is>
       </c>
     </row>
     <row r="1112">
       <c r="A1112" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1113">
       <c r="A1113" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "59ca1c3b-9f10-4420-a563-de85bfd450e3",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1114">
       <c r="A1114" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "id": "8111fdc0-a0c3-4220-8d4f-506d02e02aed",</t>
         </is>
       </c>
     </row>
     <row r="1115">
       <c r="A1115" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 3</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1116">
       <c r="A1116" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "version": 3</t>
         </is>
       </c>
     </row>
     <row r="1117">
       <c r="A1117" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1118">
       <c r="A1118" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "697585b8-3531-4640-925d-f04faec2c8b6",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1119">
       <c r="A1119" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "id": "c5f2f746-f2ee-44cb-987c-56136d5c2de1",</t>
         </is>
       </c>
     </row>
     <row r="1120">
       <c r="A1120" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 3</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1121">
       <c r="A1121" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "version": 3</t>
         </is>
       </c>
     </row>
     <row r="1122">
       <c r="A1122" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1123">
       <c r="A1123" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "515c2499-1c25-477a-be19-599581b605ff",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1124">
       <c r="A1124" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "id": "b7bc0e8e-c44c-4000-bc9b-6575a6a3f090",</t>
         </is>
       </c>
     </row>
     <row r="1125">
       <c r="A1125" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 3</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1126">
       <c r="A1126" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "version": 3</t>
         </is>
       </c>
     </row>
     <row r="1127">
       <c r="A1127" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1128">
       <c r="A1128" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "cc5edb4c-b679-4bfb-8f5c-92c60a7455fb",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1129">
       <c r="A1129" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "id": "bec5f73f-4547-4fa6-b494-4636bbb1ae62",</t>
         </is>
       </c>
     </row>
     <row r="1130">
       <c r="A1130" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 3</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1131">
       <c r="A1131" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "version": 3</t>
         </is>
       </c>
     </row>
     <row r="1132">
       <c r="A1132" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1133">
       <c r="A1133" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "75f25a9d-d846-445a-84a3-47cfd15c89ca",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1134">
       <c r="A1134" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "id": "3bcba9a4-298d-403c-bd92-b88dcd0de1e6",</t>
         </is>
       </c>
     </row>
     <row r="1135">
       <c r="A1135" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 3</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1136">
       <c r="A1136" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "version": 3</t>
         </is>
       </c>
     </row>
     <row r="1137">
       <c r="A1137" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1138">
       <c r="A1138" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "092d6bde-2841-4ef9-9d18-c01e78611952",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1139">
       <c r="A1139" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "id": "eaf1cd80-da44-4287-9129-98e9e720b8a0",</t>
         </is>
       </c>
     </row>
     <row r="1140">
       <c r="A1140" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 3</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1141">
       <c r="A1141" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "version": 3</t>
         </is>
       </c>
     </row>
     <row r="1142">
       <c r="A1142" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1143">
       <c r="A1143" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "979752dc-31f7-417a-8724-59dc251c823f",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1144">
       <c r="A1144" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "id": "6a96a1eb-21dd-4cd6-b52d-39e1d24c5c8b",</t>
         </is>
       </c>
     </row>
     <row r="1145">
       <c r="A1145" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 4</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1146">
       <c r="A1146" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "version": 4</t>
         </is>
       </c>
     </row>
     <row r="1147">
       <c r="A1147" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1148">
       <c r="A1148" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "6e9a8d48-f8fd-4609-b907-cfed7ebb2312",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1149">
       <c r="A1149" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "kind": "tp-profile",</t>
+          <t xml:space="preserve">          "id": "0a129ba1-1e8f-490f-8b33-748d6c2db1f3",</t>
         </is>
       </c>
     </row>
     <row r="1150">
       <c r="A1150" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "kind": "tp-profile",</t>
         </is>
       </c>
     </row>
     <row r="1151">
       <c r="A1151" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 3,</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1152">
       <c r="A1152" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "synthetic": false</t>
+          <t xml:space="preserve">          "version": 3,</t>
         </is>
       </c>
     </row>
     <row r="1153">
       <c r="A1153" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "synthetic": false</t>
         </is>
       </c>
     </row>
     <row r="1154">
       <c r="A1154" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1155">
       <c r="A1155" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "414fe600-3da4-49aa-818e-682e7ff12ee9",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1156">
       <c r="A1156" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "kind": "tp-rule",</t>
+          <t xml:space="preserve">          "id": "f387e7fd-fe7a-4fff-893c-f1eb47aa0ed3",</t>
         </is>
       </c>
     </row>
     <row r="1157">
       <c r="A1157" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "kind": "tp-rule",</t>
         </is>
       </c>
     </row>
     <row r="1158">
       <c r="A1158" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 3,</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1159">
       <c r="A1159" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "synthetic": false</t>
+          <t xml:space="preserve">          "version": 3,</t>
         </is>
       </c>
     </row>
     <row r="1160">
       <c r="A1160" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "synthetic": false</t>
         </is>
       </c>
     </row>
     <row r="1161">
       <c r="A1161" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1162">
       <c r="A1162" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "e5e6af42-61a4-4860-8d74-366cdf0e170c",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1163">
       <c r="A1163" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "kind": "tp-rule",</t>
+          <t xml:space="preserve">          "id": "33ed8bae-2f18-4b6a-8347-39373f58e484",</t>
         </is>
       </c>
     </row>
     <row r="1164">
       <c r="A1164" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "kind": "tp-rule",</t>
         </is>
       </c>
     </row>
     <row r="1165">
       <c r="A1165" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 3,</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1166">
       <c r="A1166" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "synthetic": false</t>
+          <t xml:space="preserve">          "version": 3,</t>
         </is>
       </c>
     </row>
     <row r="1167">
       <c r="A1167" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "synthetic": false</t>
         </is>
       </c>
     </row>
     <row r="1168">
       <c r="A1168" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1169">
       <c r="A1169" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "46495fd8-4d00-44a0-be16-adc6dbbb38c9",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1170">
       <c r="A1170" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "kind": "tp-rule",</t>
+          <t xml:space="preserve">          "id": "63b9bd2c-df96-469f-82d3-857205b0f694",</t>
         </is>
       </c>
     </row>
     <row r="1171">
       <c r="A1171" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "kind": "tp-rule",</t>
         </is>
       </c>
     </row>
     <row r="1172">
       <c r="A1172" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 3,</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1173">
       <c r="A1173" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "synthetic": false</t>
+          <t xml:space="preserve">          "version": 3,</t>
         </is>
       </c>
     </row>
     <row r="1174">
       <c r="A1174" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "synthetic": false</t>
         </is>
       </c>
     </row>
     <row r="1175">
       <c r="A1175" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1176">
       <c r="A1176" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "54f18b07-b4cf-4405-9fe2-fd35d1245db7",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1177">
       <c r="A1177" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "kind": "tp-rule",</t>
+          <t xml:space="preserve">          "id": "134ca4a1-d675-4d20-a5cc-25061178240b",</t>
         </is>
       </c>
     </row>
     <row r="1178">
       <c r="A1178" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "kind": "tp-rule",</t>
         </is>
       </c>
     </row>
     <row r="1179">
       <c r="A1179" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 3,</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1180">
       <c r="A1180" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "synthetic": false</t>
+          <t xml:space="preserve">          "version": 3,</t>
         </is>
       </c>
     </row>
     <row r="1181">
       <c r="A1181" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "synthetic": false</t>
         </is>
       </c>
     </row>
     <row r="1182">
       <c r="A1182" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1183">
       <c r="A1183" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "634078e1-cba6-4e97-b213-f6b5d5c0c729",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1184">
       <c r="A1184" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "kind": "tp-rule",</t>
+          <t xml:space="preserve">          "id": "749bfec7-47a7-4cfb-919f-6c420f9fc15f",</t>
         </is>
       </c>
     </row>
     <row r="1185">
       <c r="A1185" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "kind": "tp-rule",</t>
         </is>
       </c>
     </row>
     <row r="1186">
       <c r="A1186" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 3,</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1187">
       <c r="A1187" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "synthetic": false</t>
+          <t xml:space="preserve">          "version": 3,</t>
         </is>
       </c>
     </row>
     <row r="1188">
       <c r="A1188" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "synthetic": false</t>
         </is>
       </c>
     </row>
     <row r="1189">
       <c r="A1189" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1190">
       <c r="A1190" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "30f134e4-9320-4637-86c8-c08b0b422abb",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1191">
       <c r="A1191" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "kind": "tp-rule",</t>
+          <t xml:space="preserve">          "id": "a4399843-db68-4b86-8733-f33e5245e9c0",</t>
         </is>
       </c>
     </row>
     <row r="1192">
       <c r="A1192" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "kind": "tp-rule",</t>
         </is>
       </c>
     </row>
     <row r="1193">
       <c r="A1193" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 3,</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1194">
       <c r="A1194" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "synthetic": false</t>
+          <t xml:space="preserve">          "version": 3,</t>
         </is>
       </c>
     </row>
     <row r="1195">
       <c r="A1195" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "synthetic": false</t>
         </is>
       </c>
     </row>
     <row r="1196">
       <c r="A1196" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1197">
       <c r="A1197" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "acc88b17-2731-439a-9376-1efb4a18ff87",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1198">
       <c r="A1198" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "kind": "tp-rule",</t>
+          <t xml:space="preserve">          "id": "599f6bca-5333-467c-bbc9-5b60b04c9b3e",</t>
         </is>
       </c>
     </row>
     <row r="1199">
       <c r="A1199" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "kind": "tp-rule",</t>
         </is>
       </c>
     </row>
     <row r="1200">
       <c r="A1200" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 3,</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1201">
       <c r="A1201" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "synthetic": false</t>
+          <t xml:space="preserve">          "version": 3,</t>
         </is>
       </c>
     </row>
     <row r="1202">
       <c r="A1202" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "synthetic": false</t>
         </is>
       </c>
     </row>
     <row r="1203">
       <c r="A1203" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1204">
       <c r="A1204" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "59b42a56-53d1-4e78-ac48-7b302efed0c2",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1205">
       <c r="A1205" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "kind": "tp-localfile",</t>
+          <t xml:space="preserve">          "id": "d56ca2f7-3b45-4fc5-87b1-a298cb1f4645",</t>
         </is>
       </c>
     </row>
     <row r="1206">
       <c r="A1206" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "kind": "tp-localfile",</t>
         </is>
       </c>
     </row>
     <row r="1207">
       <c r="A1207" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 4,</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1208">
       <c r="A1208" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "synthetic": false</t>
+          <t xml:space="preserve">          "version": 4,</t>
         </is>
       </c>
     </row>
     <row r="1209">
       <c r="A1209" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "synthetic": false</t>
         </is>
       </c>
     </row>
     <row r="1210">
       <c r="A1210" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1211">
       <c r="A1211" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "caded7dc-f14d-4d3e-9103-8ceb4c8dd3ac",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1212">
       <c r="A1212" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "kind": "tp-method",</t>
+          <t xml:space="preserve">          "id": "26e3325b-a5cb-418e-8025-167c64388709",</t>
         </is>
       </c>
     </row>
     <row r="1213">
       <c r="A1213" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "kind": "ifrs-note",</t>
         </is>
       </c>
     </row>
     <row r="1214">
       <c r="A1214" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 3,</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1215">
       <c r="A1215" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "synthetic": false</t>
+          <t xml:space="preserve">          "version": 3,</t>
         </is>
       </c>
     </row>
     <row r="1216">
       <c r="A1216" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "synthetic": false</t>
         </is>
       </c>
     </row>
     <row r="1217">
       <c r="A1217" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1218">
       <c r="A1218" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "fdb9fdcd-b9c1-4573-a126-230767690bb4",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1219">
       <c r="A1219" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "kind": "tp-far",</t>
+          <t xml:space="preserve">          "id": "98678ad6-7d06-424d-ac6a-0c1f973f72ed",</t>
         </is>
       </c>
     </row>
     <row r="1220">
       <c r="A1220" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "kind": "tp-method",</t>
         </is>
       </c>
     </row>
     <row r="1221">
       <c r="A1221" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 3,</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1222">
       <c r="A1222" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "synthetic": false</t>
+          <t xml:space="preserve">          "version": 3,</t>
         </is>
       </c>
     </row>
     <row r="1223">
       <c r="A1223" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "synthetic": false</t>
         </is>
       </c>
     </row>
     <row r="1224">
       <c r="A1224" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1225">
       <c r="A1225" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "383073ea-6483-447a-8c74-fb38b6226a58",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1226">
       <c r="A1226" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "kind": "ifrs-note",</t>
+          <t xml:space="preserve">          "id": "e94f2c1e-966f-4abb-87a5-66d8467d8f35",</t>
         </is>
       </c>
     </row>
     <row r="1227">
       <c r="A1227" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "kind": "tp-far",</t>
         </is>
       </c>
     </row>
     <row r="1228">
       <c r="A1228" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 3,</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1229">
       <c r="A1229" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "synthetic": false</t>
+          <t xml:space="preserve">          "version": 3,</t>
         </is>
       </c>
     </row>
     <row r="1230">
       <c r="A1230" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "synthetic": false</t>
         </is>
       </c>
     </row>
     <row r="1231">
       <c r="A1231" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1232">
       <c r="A1232" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "64db4a8a-54e5-40a7-8654-4a16cd084ed7",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1233">
       <c r="A1233" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "kind": "tp-party",</t>
+          <t xml:space="preserve">          "id": "ad4c54ff-da6c-4474-a0d7-99c82e42ba9b",</t>
         </is>
       </c>
     </row>
     <row r="1234">
       <c r="A1234" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "kind": "tp-party",</t>
         </is>
       </c>
     </row>
     <row r="1235">
       <c r="A1235" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 3,</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1236">
       <c r="A1236" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "synthetic": true</t>
+          <t xml:space="preserve">          "version": 3,</t>
         </is>
       </c>
     </row>
     <row r="1237">
       <c r="A1237" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "synthetic": true</t>
         </is>
       </c>
     </row>
     <row r="1238">
       <c r="A1238" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1239">
       <c r="A1239" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "8d3d9472-dd0e-4e55-ac64-2e8c2cecbfc9",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1240">
       <c r="A1240" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "kind": "tp-transaction",</t>
+          <t xml:space="preserve">          "id": "249b5cc3-1aa2-4fc2-a638-fa4a21f8b192",</t>
         </is>
       </c>
     </row>
     <row r="1241">
       <c r="A1241" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "kind": "tp-transaction",</t>
         </is>
       </c>
     </row>
     <row r="1242">
       <c r="A1242" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 3,</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1243">
       <c r="A1243" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "synthetic": false</t>
+          <t xml:space="preserve">          "version": 3,</t>
         </is>
       </c>
     </row>
     <row r="1244">
       <c r="A1244" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "synthetic": false</t>
         </is>
       </c>
     </row>
     <row r="1245">
       <c r="A1245" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1246">
       <c r="A1246" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "7c6f52dd-0b10-4849-bb5b-63937e8b3f7a",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1247">
       <c r="A1247" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "kind": "tp-transaction",</t>
+          <t xml:space="preserve">          "id": "0ceeb1f1-b2a2-43ec-8d87-840f74b2dd70",</t>
         </is>
       </c>
     </row>
     <row r="1248">
       <c r="A1248" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "kind": "tp-transaction",</t>
         </is>
       </c>
     </row>
     <row r="1249">
       <c r="A1249" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 3,</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1250">
       <c r="A1250" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "synthetic": false</t>
+          <t xml:space="preserve">          "version": 3,</t>
         </is>
       </c>
     </row>
     <row r="1251">
       <c r="A1251" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "synthetic": false</t>
         </is>
       </c>
     </row>
     <row r="1252">
       <c r="A1252" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1253">
       <c r="A1253" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "26997a51-b558-43e8-a18b-8bcb0385cfe6",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1254">
       <c r="A1254" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "kind": "tp-party",</t>
+          <t xml:space="preserve">          "id": "60346b5b-473b-4889-a5da-68b017ca186b",</t>
         </is>
       </c>
     </row>
     <row r="1255">
       <c r="A1255" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "kind": "tp-party",</t>
         </is>
       </c>
     </row>
     <row r="1256">
       <c r="A1256" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 3,</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1257">
       <c r="A1257" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "synthetic": true</t>
+          <t xml:space="preserve">          "version": 3,</t>
         </is>
       </c>
     </row>
     <row r="1258">
       <c r="A1258" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "synthetic": true</t>
         </is>
       </c>
     </row>
     <row r="1259">
       <c r="A1259" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1260">
       <c r="A1260" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "5fdd6fbd-f1f1-4e9c-80b8-f76c0a7d4293",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1261">
       <c r="A1261" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "kind": "tp-relationship",</t>
+          <t xml:space="preserve">          "id": "8534d3b8-8b3a-44de-b207-57cc951802f9",</t>
         </is>
       </c>
     </row>
     <row r="1262">
       <c r="A1262" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "kind": "tp-relationship",</t>
         </is>
       </c>
     </row>
     <row r="1263">
       <c r="A1263" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 3,</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1264">
       <c r="A1264" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "synthetic": false</t>
+          <t xml:space="preserve">          "version": 3,</t>
         </is>
       </c>
     </row>
     <row r="1265">
       <c r="A1265" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "synthetic": false</t>
         </is>
       </c>
     </row>
     <row r="1266">
       <c r="A1266" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1267">
       <c r="A1267" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "634078e1-cba6-4e97-b213-f6b5d5c0c729",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1268">
       <c r="A1268" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "kind": "tp-rule",</t>
+          <t xml:space="preserve">          "id": "749bfec7-47a7-4cfb-919f-6c420f9fc15f",</t>
         </is>
       </c>
     </row>
     <row r="1269">
       <c r="A1269" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "status": "APPROVED",</t>
+          <t xml:space="preserve">          "kind": "tp-rule",</t>
         </is>
       </c>
     </row>
     <row r="1270">
       <c r="A1270" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "version": 3,</t>
+          <t xml:space="preserve">          "status": "APPROVED",</t>
         </is>
       </c>
     </row>
     <row r="1271">
       <c r="A1271" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "synthetic": false</t>
+          <t xml:space="preserve">          "version": 3,</t>
         </is>
       </c>
     </row>
     <row r="1272">
       <c r="A1272" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "synthetic": false</t>
         </is>
       </c>
     </row>
     <row r="1273">
       <c r="A1273" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1274">
       <c r="A1274" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "9f1251fa-b233-4ecd-9d23-99b681941173",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1275">
       <c r="A1275" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "type": "run",</t>
+          <t xml:space="preserve">          "id": "4728be13-cd4e-4cff-b944-aaa72314e339",</t>
         </is>
       </c>
     </row>
     <row r="1276">
       <c r="A1276" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "sha256": "4abe92101801f412f14c63a55305380d3ce93db85011148e89d4401f451873aa"</t>
+          <t xml:space="preserve">          "type": "run",</t>
         </is>
       </c>
     </row>
     <row r="1277">
       <c r="A1277" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "sha256": "bb6f6c59ca6fe7f3b2a629ba29c663b12a97df4414d9aad8e355a7a861a82292"</t>
         </is>
       </c>
     </row>
     <row r="1278">
       <c r="A1278" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1279">
       <c r="A1279" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "5361f161-7a01-4173-a92e-a24f2285d076",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1280">
       <c r="A1280" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "type": "run",</t>
+          <t xml:space="preserve">          "id": "3ad8dcc4-73bb-4757-860b-d47162b2a4cf",</t>
         </is>
       </c>
     </row>
     <row r="1281">
       <c r="A1281" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "sha256": "06691a9635e7694772fa02a48b97c4543778bd2c484c0845dab710f92384f4a5"</t>
+          <t xml:space="preserve">          "type": "run",</t>
         </is>
       </c>
     </row>
     <row r="1282">
       <c r="A1282" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "sha256": "938fe13b721d15eebe42e4915709301cad961dd4f53e781a1f34575768e4a668"</t>
         </is>
       </c>
     </row>
     <row r="1283">
       <c r="A1283" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1284">
       <c r="A1284" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "59896288-0bc4-4ef3-9045-b5dfac9177de",</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1285">
       <c r="A1285" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "type": "run",</t>
+          <t xml:space="preserve">          "id": "8a856c62-8985-46d5-913a-50057385d3f4",</t>
         </is>
       </c>
     </row>
     <row r="1286">
       <c r="A1286" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "sha256": "09fbdfee5c061267875b5ed8b9767c4068a3c86a466e2f7464e3e39c653017a6"</t>
+          <t xml:space="preserve">          "type": "run",</t>
         </is>
       </c>
     </row>
     <row r="1287">
       <c r="A1287" t="inlineStr">
         <is>
-          <t xml:space="preserve">        }</t>
+          <t xml:space="preserve">          "sha256": "11a5e9130b9b012d21bd7ed155d7173f79fb0221274b4c0d06f2ac557133d3bf"</t>
         </is>
       </c>
     </row>
     <row r="1288">
       <c r="A1288" t="inlineStr">
         <is>
-          <t xml:space="preserve">      ],</t>
+          <t xml:space="preserve">        }</t>
         </is>
       </c>
     </row>
     <row r="1289">
       <c r="A1289" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "professional_review": "DRAFT_REQUIRES_REVIEW",</t>
+          <t xml:space="preserve">      ],</t>
         </is>
       </c>
     </row>
     <row r="1290">
       <c r="A1290" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "authority_assessment": "NOT_ESTABLISHED",</t>
+          <t xml:space="preserve">      "professional_review": "DRAFT_REQUIRES_REVIEW",</t>
         </is>
       </c>
     </row>
     <row r="1291">
       <c r="A1291" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "calculated_liability": null,</t>
+          <t xml:space="preserve">      "authority_assessment": "NOT_ESTABLISHED",</t>
         </is>
       </c>
     </row>
     <row r="1292">
       <c r="A1292" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "unresolved_questions": [],</t>
+          <t xml:space="preserve">      "calculated_liability": null,</t>
         </is>
       </c>
     </row>
     <row r="1293">
       <c r="A1293" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "account_mapping_receipt": [</t>
+          <t xml:space="preserve">      "unresolved_questions": [</t>
         </is>
       </c>
     </row>
     <row r="1294">
       <c r="A1294" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">        "Synthetic benchmark population is technical test evidence, not market support for a live pricing conclusion"</t>
         </is>
       </c>
     </row>
     <row r="1295">
       <c r="A1295" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "5bcc0057-4c75-43b0-a72b-456315c7c7bc",</t>
+          <t xml:space="preserve">      ],</t>
         </is>
       </c>
     </row>
     <row r="1296">
       <c r="A1296" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "contra": false,</t>
+          <t xml:space="preserve">      "implementation_sha256": "f0117e65088943ec8e367a4d1c7c49644aaea2e1df2197768f7fe439a2e9fc4e",</t>
         </is>
       </c>
     </row>
     <row r="1297">
       <c r="A1297" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "parent_code": null,</t>
+          <t xml:space="preserve">      "account_mapping_receipt": [</t>
         </is>
       </c>
     </row>
     <row r="1298">
       <c r="A1298" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "source_group": null,</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1299">
       <c r="A1299" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "classification": null,</t>
+          <t xml:space="preserve">          "id": "71f987c2-5e78-4792-85c8-a0f350bb8c1b",</t>
         </is>
       </c>
     </row>
     <row r="1300">
       <c r="A1300" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "mapping_version": 0,</t>
+          <t xml:space="preserve">          "contra": false,</t>
         </is>
       </c>
     </row>
     <row r="1301">
       <c r="A1301" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "statement_group": null,</t>
+          <t xml:space="preserve">          "parent_code": null,</t>
         </is>
       </c>
     </row>
     <row r="1302">
       <c r="A1302" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "mapping_profile_id": null</t>
+          <t xml:space="preserve">          "source_group": null,</t>
         </is>
       </c>
     </row>
     <row r="1303">
       <c r="A1303" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "classification": null,</t>
         </is>
       </c>
     </row>
     <row r="1304">
       <c r="A1304" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">          "mapping_version": 0,</t>
         </is>
       </c>
     </row>
     <row r="1305">
       <c r="A1305" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "65d91083-9fcf-47a1-89dc-56ada0acede5",</t>
+          <t xml:space="preserve">          "statement_group": null,</t>
         </is>
       </c>
     </row>
     <row r="1306">
       <c r="A1306" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "contra": false,</t>
+          <t xml:space="preserve">          "mapping_profile_id": null</t>
         </is>
       </c>
     </row>
     <row r="1307">
       <c r="A1307" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "parent_code": null,</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1308">
       <c r="A1308" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "source_group": null,</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1309">
       <c r="A1309" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "classification": null,</t>
+          <t xml:space="preserve">          "id": "7976f107-0938-4998-be7b-8b97662b9b33",</t>
         </is>
       </c>
     </row>
     <row r="1310">
       <c r="A1310" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "mapping_version": 0,</t>
+          <t xml:space="preserve">          "contra": false,</t>
         </is>
       </c>
     </row>
     <row r="1311">
       <c r="A1311" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "statement_group": null,</t>
+          <t xml:space="preserve">          "parent_code": null,</t>
         </is>
       </c>
     </row>
     <row r="1312">
       <c r="A1312" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "mapping_profile_id": null</t>
+          <t xml:space="preserve">          "source_group": null,</t>
         </is>
       </c>
     </row>
     <row r="1313">
       <c r="A1313" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "classification": null,</t>
         </is>
       </c>
     </row>
     <row r="1314">
       <c r="A1314" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">          "mapping_version": 0,</t>
         </is>
       </c>
     </row>
     <row r="1315">
       <c r="A1315" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "a2b02874-ada3-4914-aa47-6ef905e17230",</t>
+          <t xml:space="preserve">          "statement_group": null,</t>
         </is>
       </c>
     </row>
     <row r="1316">
       <c r="A1316" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "contra": false,</t>
+          <t xml:space="preserve">          "mapping_profile_id": null</t>
         </is>
       </c>
     </row>
     <row r="1317">
       <c r="A1317" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "parent_code": null,</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1318">
       <c r="A1318" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "source_group": null,</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1319">
       <c r="A1319" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "classification": null,</t>
+          <t xml:space="preserve">          "id": "92ab2c14-847d-4b5b-8870-63f745d300cc",</t>
         </is>
       </c>
     </row>
     <row r="1320">
       <c r="A1320" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "mapping_version": 0,</t>
+          <t xml:space="preserve">          "contra": false,</t>
         </is>
       </c>
     </row>
     <row r="1321">
       <c r="A1321" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "statement_group": null,</t>
+          <t xml:space="preserve">          "parent_code": null,</t>
         </is>
       </c>
     </row>
     <row r="1322">
       <c r="A1322" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "mapping_profile_id": null</t>
+          <t xml:space="preserve">          "source_group": null,</t>
         </is>
       </c>
     </row>
     <row r="1323">
       <c r="A1323" t="inlineStr">
         <is>
-          <t xml:space="preserve">        },</t>
+          <t xml:space="preserve">          "classification": null,</t>
         </is>
       </c>
     </row>
     <row r="1324">
       <c r="A1324" t="inlineStr">
         <is>
-          <t xml:space="preserve">        {</t>
+          <t xml:space="preserve">          "mapping_version": 0,</t>
         </is>
       </c>
     </row>
     <row r="1325">
       <c r="A1325" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "e22069b3-5b24-4b32-b29e-64d279771844",</t>
+          <t xml:space="preserve">          "statement_group": null,</t>
         </is>
       </c>
     </row>
     <row r="1326">
       <c r="A1326" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "contra": false,</t>
+          <t xml:space="preserve">          "mapping_profile_id": null</t>
         </is>
       </c>
     </row>
     <row r="1327">
       <c r="A1327" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "parent_code": null,</t>
+          <t xml:space="preserve">        },</t>
         </is>
       </c>
     </row>
     <row r="1328">
       <c r="A1328" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "source_group": null,</t>
+          <t xml:space="preserve">        {</t>
         </is>
       </c>
     </row>
     <row r="1329">
       <c r="A1329" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "classification": null,</t>
+          <t xml:space="preserve">          "id": "a754e03d-faaa-434a-a71c-5d745946bda9",</t>
         </is>
       </c>
     </row>
     <row r="1330">
       <c r="A1330" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "mapping_version": 0,</t>
+          <t xml:space="preserve">          "contra": false,</t>
         </is>
       </c>
     </row>
     <row r="1331">
       <c r="A1331" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "statement_group": null,</t>
+          <t xml:space="preserve">          "parent_code": null,</t>
         </is>
       </c>
     </row>
     <row r="1332">
       <c r="A1332" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "mapping_profile_id": null</t>
+          <t xml:space="preserve">          "source_group": null,</t>
         </is>
       </c>
     </row>
     <row r="1333">
       <c r="A1333" t="inlineStr">
         <is>
-          <t xml:space="preserve">        }</t>
+          <t xml:space="preserve">          "classification": null,</t>
         </is>
       </c>
     </row>
     <row r="1334">
       <c r="A1334" t="inlineStr">
         <is>
-          <t xml:space="preserve">      ],</t>
+          <t xml:space="preserve">          "mapping_version": 0,</t>
         </is>
       </c>
     </row>
     <row r="1335">
       <c r="A1335" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "registrations_and_elections": {</t>
+          <t xml:space="preserve">          "statement_group": null,</t>
         </is>
       </c>
     </row>
     <row r="1336">
       <c r="A1336" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "sbr": null,</t>
+          <t xml:space="preserve">          "mapping_profile_id": null</t>
         </is>
       </c>
     </row>
     <row r="1337">
       <c r="A1337" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "elections": [],</t>
+          <t xml:space="preserve">        }</t>
         </is>
       </c>
     </row>
     <row r="1338">
       <c r="A1338" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "profile_id": "6e9a8d48-f8fd-4609-b907-cfed7ebb2312",</t>
+          <t xml:space="preserve">      ],</t>
         </is>
       </c>
     </row>
     <row r="1339">
       <c r="A1339" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "registration": null</t>
+          <t xml:space="preserve">      "registrations_and_elections": {</t>
         </is>
       </c>
     </row>
     <row r="1340">
       <c r="A1340" t="inlineStr">
         <is>
-          <t xml:space="preserve">      }</t>
+          <t xml:space="preserve">        "sbr": null,</t>
         </is>
       </c>
     </row>
     <row r="1341">
       <c r="A1341" t="inlineStr">
         <is>
-          <t xml:space="preserve">    },</t>
+          <t xml:space="preserve">        "elections": [],</t>
         </is>
       </c>
     </row>
     <row r="1342">
       <c r="A1342" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "annual_version": 1,</t>
+          <t xml:space="preserve">        "profile_id": "0a129ba1-1e8f-490f-8b33-748d6c2db1f3",</t>
         </is>
       </c>
     </row>
     <row r="1343">
       <c r="A1343" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "missing_sections": [],</t>
+          <t xml:space="preserve">        "registration": null,</t>
         </is>
       </c>
     </row>
     <row r="1344">
       <c r="A1344" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "software_test_data": true,</t>
+          <t xml:space="preserve">        "taxpayer_classification": null</t>
         </is>
       </c>
     </row>
     <row r="1345">
       <c r="A1345" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "financial_source_id": "c294c0ff-8c6f-4dff-8375-8f99c9058ca4",</t>
+          <t xml:space="preserve">      }</t>
         </is>
       </c>
     </row>
     <row r="1346">
       <c r="A1346" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "calculation_summaries": [</t>
+          <t xml:space="preserve">    },</t>
         </is>
       </c>
     </row>
     <row r="1347">
       <c r="A1347" t="inlineStr">
         <is>
-          <t xml:space="preserve">      {</t>
+          <t xml:space="preserve">    "annual_version": 1,</t>
         </is>
       </c>
     </row>
     <row r="1348">
       <c r="A1348" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "kind": "matrix",</t>
+          <t xml:space="preserve">    "missing_sections": [],</t>
         </is>
       </c>
     </row>
     <row r="1349">
       <c r="A1349" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "run_id": "9f1251fa-b233-4ecd-9d23-99b681941173",</t>
+          <t xml:space="preserve">    "software_test_data": true,</t>
         </is>
       </c>
     </row>
     <row r="1350">
       <c r="A1350" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "results": {</t>
+          <t xml:space="preserve">    "financial_source_id": "cf928a21-d968-43bd-af21-cbe63c33f5f4",</t>
         </is>
       </c>
     </row>
     <row r="1351">
       <c r="A1351" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "reconciled": true,</t>
+          <t xml:space="preserve">    "calculation_summaries": [</t>
         </is>
       </c>
     </row>
     <row r="1352">
       <c r="A1352" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "total_gross_values": "2800000.00000000"</t>
+          <t xml:space="preserve">      {</t>
         </is>
       </c>
     </row>
     <row r="1353">
       <c r="A1353" t="inlineStr">
         <is>
-          <t xml:space="preserve">        }</t>
+          <t xml:space="preserve">        "kind": "matrix",</t>
         </is>
       </c>
     </row>
     <row r="1354">
       <c r="A1354" t="inlineStr">
         <is>
-          <t xml:space="preserve">      },</t>
+          <t xml:space="preserve">        "run_id": "4728be13-cd4e-4cff-b944-aaa72314e339",</t>
         </is>
       </c>
     </row>
     <row r="1355">
       <c r="A1355" t="inlineStr">
         <is>
-          <t xml:space="preserve">      {</t>
+          <t xml:space="preserve">        "results": {</t>
         </is>
       </c>
     </row>
     <row r="1356">
       <c r="A1356" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "kind": "study",</t>
+          <t xml:space="preserve">          "reconciled": true,</t>
         </is>
       </c>
     </row>
     <row r="1357">
       <c r="A1357" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "run_id": "59896288-0bc4-4ef3-9045-b5dfac9177de",</t>
+          <t xml:space="preserve">          "total_gross_values": "2800000.00000000"</t>
         </is>
       </c>
     </row>
     <row r="1358">
       <c r="A1358" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "results": {</t>
+          <t xml:space="preserve">        }</t>
         </is>
       </c>
     </row>
     <row r="1359">
       <c r="A1359" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "n": 5,</t>
+          <t xml:space="preserve">      },</t>
         </is>
       </c>
     </row>
     <row r="1360">
       <c r="A1360" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "pli": "operating_margin",</t>
+          <t xml:space="preserve">      {</t>
         </is>
       </c>
     </row>
     <row r="1361">
       <c r="A1361" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "mean": "0.05600000",</t>
+          <t xml:space="preserve">        "kind": "study",</t>
         </is>
       </c>
     </row>
     <row r="1362">
       <c r="A1362" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "median": "0.05000000",</t>
+          <t xml:space="preserve">        "run_id": "8a856c62-8985-46d5-913a-50057385d3f4",</t>
         </is>
       </c>
     </row>
     <row r="1363">
       <c r="A1363" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "maximum": "0.09000000",</t>
+          <t xml:space="preserve">        "results": {</t>
         </is>
       </c>
     </row>
     <row r="1364">
       <c r="A1364" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "minimum": "0.03000000",</t>
+          <t xml:space="preserve">          "n": 5,</t>
         </is>
       </c>
     </row>
     <row r="1365">
       <c r="A1365" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "purpose": "profitability",</t>
+          <t xml:space="preserve">          "pli": "operating_margin",</t>
         </is>
       </c>
     </row>
     <row r="1366">
       <c r="A1366" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "currency": "AED",</t>
+          <t xml:space="preserve">          "mean": "0.05600000",</t>
         </is>
       </c>
     </row>
     <row r="1367">
       <c r="A1367" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "synthetic": true,</t>
+          <t xml:space="preserve">          "median": "0.05000000",</t>
         </is>
       </c>
     </row>
     <row r="1368">
       <c r="A1368" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "lower_quartile": "0.04000000",</t>
+          <t xml:space="preserve">          "maximum": "0.09000000",</t>
         </is>
       </c>
     </row>
     <row r="1369">
       <c r="A1369" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "upper_quartile": "0.07000000",</t>
+          <t xml:space="preserve">          "minimum": "0.03000000",</t>
         </is>
       </c>
     </row>
     <row r="1370">
       <c r="A1370" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "selected_target": null</t>
+          <t xml:space="preserve">          "purpose": "profitability",</t>
         </is>
       </c>
     </row>
     <row r="1371">
       <c r="A1371" t="inlineStr">
         <is>
-          <t xml:space="preserve">        }</t>
+          <t xml:space="preserve">          "currency": "AED",</t>
         </is>
       </c>
     </row>
     <row r="1372">
       <c r="A1372" t="inlineStr">
         <is>
-          <t xml:space="preserve">      }</t>
+          <t xml:space="preserve">          "synthetic": true,</t>
         </is>
       </c>
     </row>
     <row r="1373">
       <c r="A1373" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ],</t>
+          <t xml:space="preserve">          "lower_quartile": "0.04000000",</t>
         </is>
       </c>
     </row>
     <row r="1374">
       <c r="A1374" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "financial_reconciliation_run_id": "5361f161-7a01-4173-a92e-a24f2285d076"</t>
+          <t xml:space="preserve">          "upper_quartile": "0.07000000",</t>
         </is>
       </c>
     </row>
     <row r="1375">
       <c r="A1375" t="inlineStr">
         <is>
-          <t xml:space="preserve">  }</t>
+          <t xml:space="preserve">          "selected_target": null</t>
         </is>
       </c>
     </row>
     <row r="1376">
       <c r="A1376" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        }</t>
+        </is>
+      </c>
+    </row>
+    <row r="1377">
+      <c r="A1377" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      }</t>
+        </is>
+      </c>
+    </row>
+    <row r="1378">
+      <c r="A1378" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ],</t>
+        </is>
+      </c>
+    </row>
+    <row r="1379">
+      <c r="A1379" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    "financial_reconciliation_run_id": "3ad8dcc4-73bb-4757-860b-d47162b2a4cf"</t>
+        </is>
+      </c>
+    </row>
+    <row r="1380">
+      <c r="A1380" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  }</t>
+        </is>
+      </c>
+    </row>
+    <row r="1381">
+      <c r="A1381" t="inlineStr">
         <is>
           <t>}</t>
         </is>

</xml_diff>

<commit_message>
Implement country workflows, accounting extensions and ML foundation
</commit_message>
<xml_diff>
--- a/docs/phase-8/export-evidence/synthetic-localfile.xlsx
+++ b/docs/phase-8/export-evidence/synthetic-localfile.xlsx
@@ -483,7 +483,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>342f126e-d16f-4cac-bec8-2c13a4833ba3 / auditos-tp/1.0</t>
+          <t>0258664f-47b6-46cf-ba0d-4b0c06ec4f67 / auditos-tp/1.0</t>
         </is>
       </c>
     </row>
@@ -507,7 +507,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>099843472321e21f9215341804f6d400dbc19e6b8e845127925240acdd6fbd05</t>
+          <t>a489c9f48f7cccb23436466168f765d8c10bbf8e97b0391990aa24061a410ac9</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>26e3325b-a5cb-418e-8025-167c64388709</t>
+          <t>3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0</t>
         </is>
       </c>
     </row>
@@ -605,7 +605,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>26e3325b-a5cb-418e-8025-167c64388709</t>
+          <t>3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0</t>
         </is>
       </c>
     </row>
@@ -636,7 +636,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>26e3325b-a5cb-418e-8025-167c64388709</t>
+          <t>3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0</t>
         </is>
       </c>
     </row>
@@ -667,7 +667,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>26e3325b-a5cb-418e-8025-167c64388709</t>
+          <t>3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0</t>
         </is>
       </c>
     </row>
@@ -698,7 +698,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>26e3325b-a5cb-418e-8025-167c64388709</t>
+          <t>3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0</t>
         </is>
       </c>
     </row>
@@ -729,7 +729,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>26e3325b-a5cb-418e-8025-167c64388709</t>
+          <t>3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0</t>
         </is>
       </c>
     </row>
@@ -741,7 +741,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>4728be13-cd4e-4cff-b944-aaa72314e339</t>
+          <t>3e0e7d7b-c078-41f1-887b-adbd588c0d57</t>
         </is>
       </c>
     </row>
@@ -772,7 +772,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>26e3325b-a5cb-418e-8025-167c64388709</t>
+          <t>3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>e94f2c1e-966f-4abb-87a5-66d8467d8f35</t>
+          <t>30e11100-a98b-4418-806b-7b0062760904</t>
         </is>
       </c>
     </row>
@@ -834,7 +834,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>98678ad6-7d06-424d-ac6a-0c1f973f72ed</t>
+          <t>8f8e7a1e-a7bc-4812-91f0-d76c99dcf630</t>
         </is>
       </c>
     </row>
@@ -865,7 +865,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>26e3325b-a5cb-418e-8025-167c64388709</t>
+          <t>3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0</t>
         </is>
       </c>
     </row>
@@ -896,7 +896,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>26e3325b-a5cb-418e-8025-167c64388709</t>
+          <t>3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>8a856c62-8985-46d5-913a-50057385d3f4</t>
+          <t>4852218e-f3f3-4ac7-93dc-f5a525cf96c5</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>26e3325b-a5cb-418e-8025-167c64388709</t>
+          <t>3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0</t>
         </is>
       </c>
     </row>
@@ -970,7 +970,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>26e3325b-a5cb-418e-8025-167c64388709</t>
+          <t>3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>26e3325b-a5cb-418e-8025-167c64388709</t>
+          <t>3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0</t>
         </is>
       </c>
     </row>
@@ -1013,7 +1013,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>4728be13-cd4e-4cff-b944-aaa72314e339</t>
+          <t>3e0e7d7b-c078-41f1-887b-adbd588c0d57</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1049,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>8a856c62-8985-46d5-913a-50057385d3f4</t>
+          <t>4852218e-f3f3-4ac7-93dc-f5a525cf96c5</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "5d6b30ea-667e-4f01-8d3b-219507024f74",</t>
+          <t xml:space="preserve">    "id": "7c922cee-c000-47e0-9e18-e1c67f256d14",</t>
         </is>
       </c>
     </row>
@@ -1266,7 +1266,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "5151ae5a-ab3c-4239-9116-57444f6179d2",</t>
+          <t xml:space="preserve">    "id": "fdccd6c0-ab9a-4d7c-9480-1cb36f6b8659",</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1301,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "07be194f-aefb-4021-891f-f42b00d1d380",</t>
+          <t xml:space="preserve">    "id": "1e5812ed-4402-4b7f-b92c-49b6428c6ec2",</t>
         </is>
       </c>
     </row>
@@ -1336,7 +1336,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "26e3325b-a5cb-418e-8025-167c64388709",</t>
+          <t xml:space="preserve">    "id": "3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0",</t>
         </is>
       </c>
     </row>
@@ -1371,7 +1371,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "8111fdc0-a0c3-4220-8d4f-506d02e02aed",</t>
+          <t xml:space="preserve">    "id": "2205c942-8a3b-4df5-8539-6470ac261cc8",</t>
         </is>
       </c>
     </row>
@@ -1406,7 +1406,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "c5f2f746-f2ee-44cb-987c-56136d5c2de1",</t>
+          <t xml:space="preserve">    "id": "b243bb9b-6bbb-4c0c-bd5b-5d1c04d48f06",</t>
         </is>
       </c>
     </row>
@@ -1441,7 +1441,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "b7bc0e8e-c44c-4000-bc9b-6575a6a3f090",</t>
+          <t xml:space="preserve">    "id": "fb515fbf-b17a-4def-9671-dd74a6b9e094",</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1476,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "bec5f73f-4547-4fa6-b494-4636bbb1ae62",</t>
+          <t xml:space="preserve">    "id": "6f8b9d96-c0ae-436b-85c0-339a0c4aa4d9",</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1511,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "3bcba9a4-298d-403c-bd92-b88dcd0de1e6",</t>
+          <t xml:space="preserve">    "id": "fa126d00-0e5e-42e4-b043-4938f4c66cd9",</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "eaf1cd80-da44-4287-9129-98e9e720b8a0",</t>
+          <t xml:space="preserve">    "id": "51c8f8a1-5c9a-4d37-8453-a21c548c739d",</t>
         </is>
       </c>
     </row>
@@ -1581,7 +1581,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "6a96a1eb-21dd-4cd6-b52d-39e1d24c5c8b",</t>
+          <t xml:space="preserve">    "id": "f17b2344-beab-4a85-ac9c-2316b5015994",</t>
         </is>
       </c>
     </row>
@@ -1616,7 +1616,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "0a129ba1-1e8f-490f-8b33-748d6c2db1f3",</t>
+          <t xml:space="preserve">    "id": "dbf32166-b457-4c44-a482-333f013e9541",</t>
         </is>
       </c>
     </row>
@@ -1665,7 +1665,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "f387e7fd-fe7a-4fff-893c-f1eb47aa0ed3",</t>
+          <t xml:space="preserve">    "id": "4a227430-8782-4779-a651-e7231042a27a",</t>
         </is>
       </c>
     </row>
@@ -1714,7 +1714,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "33ed8bae-2f18-4b6a-8347-39373f58e484",</t>
+          <t xml:space="preserve">    "id": "8c530841-0422-4d7a-8873-512cc840211e",</t>
         </is>
       </c>
     </row>
@@ -1763,7 +1763,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "63b9bd2c-df96-469f-82d3-857205b0f694",</t>
+          <t xml:space="preserve">    "id": "35b21af8-1e1c-4fe3-b402-6c26e3f289b4",</t>
         </is>
       </c>
     </row>
@@ -1812,7 +1812,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "134ca4a1-d675-4d20-a5cc-25061178240b",</t>
+          <t xml:space="preserve">    "id": "3cc2f1e2-0cb1-4fa3-841c-274d6be8fe8b",</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "749bfec7-47a7-4cfb-919f-6c420f9fc15f",</t>
+          <t xml:space="preserve">    "id": "7b5603f4-6138-4607-af70-515610f0da73",</t>
         </is>
       </c>
     </row>
@@ -1910,7 +1910,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "a4399843-db68-4b86-8733-f33e5245e9c0",</t>
+          <t xml:space="preserve">    "id": "6d9f0a74-5cfe-4f26-b921-cb4c62d57f4b",</t>
         </is>
       </c>
     </row>
@@ -1959,7 +1959,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "599f6bca-5333-467c-bbc9-5b60b04c9b3e",</t>
+          <t xml:space="preserve">    "id": "b8285a20-103d-42c9-9cd0-eeadffc93ab1",</t>
         </is>
       </c>
     </row>
@@ -2008,7 +2008,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "d56ca2f7-3b45-4fc5-87b1-a298cb1f4645",</t>
+          <t xml:space="preserve">    "id": "b39363ca-4043-4e47-924e-d492e6537e59",</t>
         </is>
       </c>
     </row>
@@ -2057,14 +2057,14 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "26e3325b-a5cb-418e-8025-167c64388709",</t>
+          <t xml:space="preserve">    "id": "30e11100-a98b-4418-806b-7b0062760904",</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "kind": "ifrs-note",</t>
+          <t xml:space="preserve">    "kind": "tp-far",</t>
         </is>
       </c>
     </row>
@@ -2106,7 +2106,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "98678ad6-7d06-424d-ac6a-0c1f973f72ed",</t>
+          <t xml:space="preserve">    "id": "8f8e7a1e-a7bc-4812-91f0-d76c99dcf630",</t>
         </is>
       </c>
     </row>
@@ -2155,14 +2155,14 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "e94f2c1e-966f-4abb-87a5-66d8467d8f35",</t>
+          <t xml:space="preserve">    "id": "3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0",</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "kind": "tp-far",</t>
+          <t xml:space="preserve">    "kind": "ifrs-note",</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2204,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "ad4c54ff-da6c-4474-a0d7-99c82e42ba9b",</t>
+          <t xml:space="preserve">    "id": "78c8e4a2-30a6-4043-ab30-8f30b5206b63",</t>
         </is>
       </c>
     </row>
@@ -2253,7 +2253,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "249b5cc3-1aa2-4fc2-a638-fa4a21f8b192",</t>
+          <t xml:space="preserve">    "id": "1fdbf156-cf26-4343-ae8e-35306c4317d4",</t>
         </is>
       </c>
     </row>
@@ -2302,7 +2302,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "0ceeb1f1-b2a2-43ec-8d87-840f74b2dd70",</t>
+          <t xml:space="preserve">    "id": "4942fe08-8c8c-47a8-8d93-b25684055404",</t>
         </is>
       </c>
     </row>
@@ -2351,7 +2351,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "60346b5b-473b-4889-a5da-68b017ca186b",</t>
+          <t xml:space="preserve">    "id": "be3f8a86-2ec4-4216-a9d5-aad320edb4a7",</t>
         </is>
       </c>
     </row>
@@ -2400,7 +2400,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "8534d3b8-8b3a-44de-b207-57cc951802f9",</t>
+          <t xml:space="preserve">    "id": "3cc9dc57-ce14-47b2-afe4-053e2ddf3ce3",</t>
         </is>
       </c>
     </row>
@@ -2449,7 +2449,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "749bfec7-47a7-4cfb-919f-6c420f9fc15f",</t>
+          <t xml:space="preserve">    "id": "7b5603f4-6138-4607-af70-515610f0da73",</t>
         </is>
       </c>
     </row>
@@ -2498,7 +2498,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "4728be13-cd4e-4cff-b944-aaa72314e339",</t>
+          <t xml:space="preserve">    "id": "a068f299-a348-4b3c-bdd6-72eddf9ad9c2",</t>
         </is>
       </c>
     </row>
@@ -2512,7 +2512,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "sha256": "bb6f6c59ca6fe7f3b2a629ba29c663b12a97df4414d9aad8e355a7a861a82292"</t>
+          <t xml:space="preserve">    "sha256": "bf71045089aa949cc8b15a40099a37437bd3959c1aabfcf02d7ab34f63fc6b76"</t>
         </is>
       </c>
     </row>
@@ -2533,7 +2533,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "3ad8dcc4-73bb-4757-860b-d47162b2a4cf",</t>
+          <t xml:space="preserve">    "id": "3e0e7d7b-c078-41f1-887b-adbd588c0d57",</t>
         </is>
       </c>
     </row>
@@ -2547,7 +2547,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "sha256": "938fe13b721d15eebe42e4915709301cad961dd4f53e781a1f34575768e4a668"</t>
+          <t xml:space="preserve">    "sha256": "d6cb1126efd9719296f6f085bf132532baa9572aeb6618772d51dc7d65e6e228"</t>
         </is>
       </c>
     </row>
@@ -2568,7 +2568,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "id": "8a856c62-8985-46d5-913a-50057385d3f4",</t>
+          <t xml:space="preserve">    "id": "4852218e-f3f3-4ac7-93dc-f5a525cf96c5",</t>
         </is>
       </c>
     </row>
@@ -2582,7 +2582,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "sha256": "11a5e9130b9b012d21bd7ed155d7173f79fb0221274b4c0d06f2ac557133d3bf"</t>
+          <t xml:space="preserve">    "sha256": "384d550fadd1c9918ea31b0df66c48fd83576321952e40c92268e587b5166633"</t>
         </is>
       </c>
     </row>
@@ -2627,14 +2627,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  "id": "342f126e-d16f-4cac-bec8-2c13a4833ba3",</t>
+          <t xml:space="preserve">  "id": "0258664f-47b6-46cf-ba0d-4b0c06ec4f67",</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  "sha256": "099843472321e21f9215341804f6d400dbc19e6b8e845127925240acdd6fbd05",</t>
+          <t xml:space="preserve">  "sha256": "a489c9f48f7cccb23436466168f765d8c10bbf8e97b0391990aa24061a410ac9",</t>
         </is>
       </c>
     </row>
@@ -2655,14 +2655,14 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  "prepared_by": "368c7cfa-ac0d-4a06-a71c-247c923c7eee",</t>
+          <t xml:space="preserve">  "prepared_by": "b32f2275-94b0-48a5-93ac-9d374278d9e1",</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  "created_at": "2026-10-24 18:34:29.653566+00:00",</t>
+          <t xml:space="preserve">  "created_at": "2026-10-24 18:43:59.521417+00:00",</t>
         </is>
       </c>
     </row>
@@ -2683,14 +2683,14 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "record_id": "d56ca2f7-3b45-4fc5-87b1-a298cb1f4645",</t>
+          <t xml:space="preserve">    "record_id": "b39363ca-4043-4e47-924e-d492e6537e59",</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "profile_id": "0a129ba1-1e8f-490f-8b33-748d6c2db1f3"</t>
+          <t xml:space="preserve">    "profile_id": "dbf32166-b457-4c44-a482-333f013e9541"</t>
         </is>
       </c>
     </row>
@@ -2718,7 +2718,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "5d6b30ea-667e-4f01-8d3b-219507024f74",</t>
+          <t xml:space="preserve">      "id": "7c922cee-c000-47e0-9e18-e1c67f256d14",</t>
         </is>
       </c>
     </row>
@@ -2753,7 +2753,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "5151ae5a-ab3c-4239-9116-57444f6179d2",</t>
+          <t xml:space="preserve">      "id": "fdccd6c0-ab9a-4d7c-9480-1cb36f6b8659",</t>
         </is>
       </c>
     </row>
@@ -2788,7 +2788,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "07be194f-aefb-4021-891f-f42b00d1d380",</t>
+          <t xml:space="preserve">      "id": "1e5812ed-4402-4b7f-b92c-49b6428c6ec2",</t>
         </is>
       </c>
     </row>
@@ -2823,7 +2823,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "26e3325b-a5cb-418e-8025-167c64388709",</t>
+          <t xml:space="preserve">      "id": "3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0",</t>
         </is>
       </c>
     </row>
@@ -2858,7 +2858,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "8111fdc0-a0c3-4220-8d4f-506d02e02aed",</t>
+          <t xml:space="preserve">      "id": "2205c942-8a3b-4df5-8539-6470ac261cc8",</t>
         </is>
       </c>
     </row>
@@ -2893,7 +2893,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "c5f2f746-f2ee-44cb-987c-56136d5c2de1",</t>
+          <t xml:space="preserve">      "id": "b243bb9b-6bbb-4c0c-bd5b-5d1c04d48f06",</t>
         </is>
       </c>
     </row>
@@ -2928,7 +2928,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "b7bc0e8e-c44c-4000-bc9b-6575a6a3f090",</t>
+          <t xml:space="preserve">      "id": "fb515fbf-b17a-4def-9671-dd74a6b9e094",</t>
         </is>
       </c>
     </row>
@@ -2963,7 +2963,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "bec5f73f-4547-4fa6-b494-4636bbb1ae62",</t>
+          <t xml:space="preserve">      "id": "6f8b9d96-c0ae-436b-85c0-339a0c4aa4d9",</t>
         </is>
       </c>
     </row>
@@ -2998,7 +2998,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "3bcba9a4-298d-403c-bd92-b88dcd0de1e6",</t>
+          <t xml:space="preserve">      "id": "fa126d00-0e5e-42e4-b043-4938f4c66cd9",</t>
         </is>
       </c>
     </row>
@@ -3033,7 +3033,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "eaf1cd80-da44-4287-9129-98e9e720b8a0",</t>
+          <t xml:space="preserve">      "id": "51c8f8a1-5c9a-4d37-8453-a21c548c739d",</t>
         </is>
       </c>
     </row>
@@ -3068,7 +3068,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "6a96a1eb-21dd-4cd6-b52d-39e1d24c5c8b",</t>
+          <t xml:space="preserve">      "id": "f17b2344-beab-4a85-ac9c-2316b5015994",</t>
         </is>
       </c>
     </row>
@@ -3103,7 +3103,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "0a129ba1-1e8f-490f-8b33-748d6c2db1f3",</t>
+          <t xml:space="preserve">      "id": "dbf32166-b457-4c44-a482-333f013e9541",</t>
         </is>
       </c>
     </row>
@@ -3152,7 +3152,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "f387e7fd-fe7a-4fff-893c-f1eb47aa0ed3",</t>
+          <t xml:space="preserve">      "id": "4a227430-8782-4779-a651-e7231042a27a",</t>
         </is>
       </c>
     </row>
@@ -3201,7 +3201,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "33ed8bae-2f18-4b6a-8347-39373f58e484",</t>
+          <t xml:space="preserve">      "id": "8c530841-0422-4d7a-8873-512cc840211e",</t>
         </is>
       </c>
     </row>
@@ -3250,7 +3250,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "63b9bd2c-df96-469f-82d3-857205b0f694",</t>
+          <t xml:space="preserve">      "id": "35b21af8-1e1c-4fe3-b402-6c26e3f289b4",</t>
         </is>
       </c>
     </row>
@@ -3299,7 +3299,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "134ca4a1-d675-4d20-a5cc-25061178240b",</t>
+          <t xml:space="preserve">      "id": "3cc2f1e2-0cb1-4fa3-841c-274d6be8fe8b",</t>
         </is>
       </c>
     </row>
@@ -3348,7 +3348,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "749bfec7-47a7-4cfb-919f-6c420f9fc15f",</t>
+          <t xml:space="preserve">      "id": "7b5603f4-6138-4607-af70-515610f0da73",</t>
         </is>
       </c>
     </row>
@@ -3397,7 +3397,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "a4399843-db68-4b86-8733-f33e5245e9c0",</t>
+          <t xml:space="preserve">      "id": "6d9f0a74-5cfe-4f26-b921-cb4c62d57f4b",</t>
         </is>
       </c>
     </row>
@@ -3446,7 +3446,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "599f6bca-5333-467c-bbc9-5b60b04c9b3e",</t>
+          <t xml:space="preserve">      "id": "b8285a20-103d-42c9-9cd0-eeadffc93ab1",</t>
         </is>
       </c>
     </row>
@@ -3495,7 +3495,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "d56ca2f7-3b45-4fc5-87b1-a298cb1f4645",</t>
+          <t xml:space="preserve">      "id": "b39363ca-4043-4e47-924e-d492e6537e59",</t>
         </is>
       </c>
     </row>
@@ -3544,14 +3544,14 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "26e3325b-a5cb-418e-8025-167c64388709",</t>
+          <t xml:space="preserve">      "id": "30e11100-a98b-4418-806b-7b0062760904",</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "kind": "ifrs-note",</t>
+          <t xml:space="preserve">      "kind": "tp-far",</t>
         </is>
       </c>
     </row>
@@ -3593,7 +3593,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "98678ad6-7d06-424d-ac6a-0c1f973f72ed",</t>
+          <t xml:space="preserve">      "id": "8f8e7a1e-a7bc-4812-91f0-d76c99dcf630",</t>
         </is>
       </c>
     </row>
@@ -3642,14 +3642,14 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "e94f2c1e-966f-4abb-87a5-66d8467d8f35",</t>
+          <t xml:space="preserve">      "id": "3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0",</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "kind": "tp-far",</t>
+          <t xml:space="preserve">      "kind": "ifrs-note",</t>
         </is>
       </c>
     </row>
@@ -3691,7 +3691,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "ad4c54ff-da6c-4474-a0d7-99c82e42ba9b",</t>
+          <t xml:space="preserve">      "id": "78c8e4a2-30a6-4043-ab30-8f30b5206b63",</t>
         </is>
       </c>
     </row>
@@ -3740,7 +3740,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "249b5cc3-1aa2-4fc2-a638-fa4a21f8b192",</t>
+          <t xml:space="preserve">      "id": "1fdbf156-cf26-4343-ae8e-35306c4317d4",</t>
         </is>
       </c>
     </row>
@@ -3789,7 +3789,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "0ceeb1f1-b2a2-43ec-8d87-840f74b2dd70",</t>
+          <t xml:space="preserve">      "id": "4942fe08-8c8c-47a8-8d93-b25684055404",</t>
         </is>
       </c>
     </row>
@@ -3838,7 +3838,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "60346b5b-473b-4889-a5da-68b017ca186b",</t>
+          <t xml:space="preserve">      "id": "be3f8a86-2ec4-4216-a9d5-aad320edb4a7",</t>
         </is>
       </c>
     </row>
@@ -3887,7 +3887,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "8534d3b8-8b3a-44de-b207-57cc951802f9",</t>
+          <t xml:space="preserve">      "id": "3cc9dc57-ce14-47b2-afe4-053e2ddf3ce3",</t>
         </is>
       </c>
     </row>
@@ -3936,7 +3936,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "749bfec7-47a7-4cfb-919f-6c420f9fc15f",</t>
+          <t xml:space="preserve">      "id": "7b5603f4-6138-4607-af70-515610f0da73",</t>
         </is>
       </c>
     </row>
@@ -3985,7 +3985,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "4728be13-cd4e-4cff-b944-aaa72314e339",</t>
+          <t xml:space="preserve">      "id": "a068f299-a348-4b3c-bdd6-72eddf9ad9c2",</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "sha256": "bb6f6c59ca6fe7f3b2a629ba29c663b12a97df4414d9aad8e355a7a861a82292"</t>
+          <t xml:space="preserve">      "sha256": "bf71045089aa949cc8b15a40099a37437bd3959c1aabfcf02d7ab34f63fc6b76"</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "3ad8dcc4-73bb-4757-860b-d47162b2a4cf",</t>
+          <t xml:space="preserve">      "id": "3e0e7d7b-c078-41f1-887b-adbd588c0d57",</t>
         </is>
       </c>
     </row>
@@ -4034,7 +4034,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "sha256": "938fe13b721d15eebe42e4915709301cad961dd4f53e781a1f34575768e4a668"</t>
+          <t xml:space="preserve">      "sha256": "d6cb1126efd9719296f6f085bf132532baa9572aeb6618772d51dc7d65e6e228"</t>
         </is>
       </c>
     </row>
@@ -4055,7 +4055,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "id": "8a856c62-8985-46d5-913a-50057385d3f4",</t>
+          <t xml:space="preserve">      "id": "4852218e-f3f3-4ac7-93dc-f5a525cf96c5",</t>
         </is>
       </c>
     </row>
@@ -4069,7 +4069,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "sha256": "11a5e9130b9b012d21bd7ed155d7173f79fb0221274b4c0d06f2ac557133d3bf"</t>
+          <t xml:space="preserve">      "sha256": "384d550fadd1c9918ea31b0df66c48fd83576321952e40c92268e587b5166633"</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t xml:space="preserve">            "da75be6b-463d-44e4-8dc4-1e26094a7ff7"</t>
+          <t xml:space="preserve">            "d6a38fec-06bb-4142-be24-a5abb76c6d31"</t>
         </is>
       </c>
     </row>
@@ -4349,7 +4349,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "rule_record_id": "f387e7fd-fe7a-4fff-893c-f1eb47aa0ed3",</t>
+          <t xml:space="preserve">        "rule_record_id": "4a227430-8782-4779-a651-e7231042a27a",</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t xml:space="preserve">            "da75be6b-463d-44e4-8dc4-1e26094a7ff7"</t>
+          <t xml:space="preserve">            "d6a38fec-06bb-4142-be24-a5abb76c6d31"</t>
         </is>
       </c>
     </row>
@@ -4706,7 +4706,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "rule_record_id": "33ed8bae-2f18-4b6a-8347-39373f58e484",</t>
+          <t xml:space="preserve">        "rule_record_id": "8c530841-0422-4d7a-8873-512cc840211e",</t>
         </is>
       </c>
     </row>
@@ -5014,7 +5014,7 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t xml:space="preserve">            "da75be6b-463d-44e4-8dc4-1e26094a7ff7"</t>
+          <t xml:space="preserve">            "d6a38fec-06bb-4142-be24-a5abb76c6d31"</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "rule_record_id": "63b9bd2c-df96-469f-82d3-857205b0f694",</t>
+          <t xml:space="preserve">        "rule_record_id": "35b21af8-1e1c-4fe3-b402-6c26e3f289b4",</t>
         </is>
       </c>
     </row>
@@ -5399,7 +5399,7 @@
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t xml:space="preserve">            "da75be6b-463d-44e4-8dc4-1e26094a7ff7"</t>
+          <t xml:space="preserve">            "d6a38fec-06bb-4142-be24-a5abb76c6d31"</t>
         </is>
       </c>
     </row>
@@ -5434,7 +5434,7 @@
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "rule_record_id": "134ca4a1-d675-4d20-a5cc-25061178240b",</t>
+          <t xml:space="preserve">        "rule_record_id": "3cc2f1e2-0cb1-4fa3-841c-274d6be8fe8b",</t>
         </is>
       </c>
     </row>
@@ -5749,7 +5749,7 @@
     <row r="448">
       <c r="A448" t="inlineStr">
         <is>
-          <t xml:space="preserve">            "da75be6b-463d-44e4-8dc4-1e26094a7ff7"</t>
+          <t xml:space="preserve">            "d6a38fec-06bb-4142-be24-a5abb76c6d31"</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "rule_record_id": "749bfec7-47a7-4cfb-919f-6c420f9fc15f",</t>
+          <t xml:space="preserve">        "rule_record_id": "7b5603f4-6138-4607-af70-515610f0da73",</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
     <row r="498">
       <c r="A498" t="inlineStr">
         <is>
-          <t xml:space="preserve">            "da75be6b-463d-44e4-8dc4-1e26094a7ff7"</t>
+          <t xml:space="preserve">            "d6a38fec-06bb-4142-be24-a5abb76c6d31"</t>
         </is>
       </c>
     </row>
@@ -6134,7 +6134,7 @@
     <row r="503">
       <c r="A503" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "rule_record_id": "a4399843-db68-4b86-8733-f33e5245e9c0",</t>
+          <t xml:space="preserve">        "rule_record_id": "6d9f0a74-5cfe-4f26-b921-cb4c62d57f4b",</t>
         </is>
       </c>
     </row>
@@ -6449,7 +6449,7 @@
     <row r="548">
       <c r="A548" t="inlineStr">
         <is>
-          <t xml:space="preserve">            "da75be6b-463d-44e4-8dc4-1e26094a7ff7"</t>
+          <t xml:space="preserve">            "d6a38fec-06bb-4142-be24-a5abb76c6d31"</t>
         </is>
       </c>
     </row>
@@ -6484,7 +6484,7 @@
     <row r="553">
       <c r="A553" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "rule_record_id": "599f6bca-5333-467c-bbc9-5b60b04c9b3e",</t>
+          <t xml:space="preserve">        "rule_record_id": "b8285a20-103d-42c9-9cd0-eeadffc93ab1",</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
     <row r="576">
       <c r="A576" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "26e3325b-a5cb-418e-8025-167c64388709"</t>
+          <t xml:space="preserve">          "3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0"</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
     <row r="585">
       <c r="A585" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "26e3325b-a5cb-418e-8025-167c64388709"</t>
+          <t xml:space="preserve">          "3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0"</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
     <row r="594">
       <c r="A594" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "26e3325b-a5cb-418e-8025-167c64388709"</t>
+          <t xml:space="preserve">          "3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0"</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
     <row r="603">
       <c r="A603" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "26e3325b-a5cb-418e-8025-167c64388709"</t>
+          <t xml:space="preserve">          "3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0"</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
     <row r="612">
       <c r="A612" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "26e3325b-a5cb-418e-8025-167c64388709"</t>
+          <t xml:space="preserve">          "3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0"</t>
         </is>
       </c>
     </row>
@@ -6946,7 +6946,7 @@
     <row r="619">
       <c r="A619" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "4728be13-cd4e-4cff-b944-aaa72314e339"</t>
+          <t xml:space="preserve">          "3e0e7d7b-c078-41f1-887b-adbd588c0d57"</t>
         </is>
       </c>
     </row>
@@ -6974,7 +6974,7 @@
     <row r="623">
       <c r="A623" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "26e3325b-a5cb-418e-8025-167c64388709"</t>
+          <t xml:space="preserve">          "3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0"</t>
         </is>
       </c>
     </row>
@@ -7037,7 +7037,7 @@
     <row r="632">
       <c r="A632" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "26e3325b-a5cb-418e-8025-167c64388709"</t>
+          <t xml:space="preserve">          "3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0"</t>
         </is>
       </c>
     </row>
@@ -7100,7 +7100,7 @@
     <row r="641">
       <c r="A641" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "e94f2c1e-966f-4abb-87a5-66d8467d8f35"</t>
+          <t xml:space="preserve">          "30e11100-a98b-4418-806b-7b0062760904"</t>
         </is>
       </c>
     </row>
@@ -7163,7 +7163,7 @@
     <row r="650">
       <c r="A650" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "98678ad6-7d06-424d-ac6a-0c1f973f72ed"</t>
+          <t xml:space="preserve">          "8f8e7a1e-a7bc-4812-91f0-d76c99dcf630"</t>
         </is>
       </c>
     </row>
@@ -7226,7 +7226,7 @@
     <row r="659">
       <c r="A659" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "26e3325b-a5cb-418e-8025-167c64388709"</t>
+          <t xml:space="preserve">          "3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0"</t>
         </is>
       </c>
     </row>
@@ -7275,7 +7275,7 @@
     <row r="666">
       <c r="A666" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "8a856c62-8985-46d5-913a-50057385d3f4"</t>
+          <t xml:space="preserve">          "4852218e-f3f3-4ac7-93dc-f5a525cf96c5"</t>
         </is>
       </c>
     </row>
@@ -7303,7 +7303,7 @@
     <row r="670">
       <c r="A670" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "26e3325b-a5cb-418e-8025-167c64388709"</t>
+          <t xml:space="preserve">          "3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0"</t>
         </is>
       </c>
     </row>
@@ -7366,7 +7366,7 @@
     <row r="679">
       <c r="A679" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "26e3325b-a5cb-418e-8025-167c64388709"</t>
+          <t xml:space="preserve">          "3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0"</t>
         </is>
       </c>
     </row>
@@ -7429,7 +7429,7 @@
     <row r="688">
       <c r="A688" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "26e3325b-a5cb-418e-8025-167c64388709"</t>
+          <t xml:space="preserve">          "3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0"</t>
         </is>
       </c>
     </row>
@@ -7492,7 +7492,7 @@
     <row r="697">
       <c r="A697" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "26e3325b-a5cb-418e-8025-167c64388709"</t>
+          <t xml:space="preserve">          "3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0"</t>
         </is>
       </c>
     </row>
@@ -7527,7 +7527,7 @@
     <row r="702">
       <c r="A702" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "entity_id": "26047f96-aba9-4e5f-97eb-a04d18c3e2ce",</t>
+          <t xml:space="preserve">    "entity_id": "c2c5b835-808e-413d-a637-67ece499bbdf",</t>
         </is>
       </c>
     </row>
@@ -7548,7 +7548,7 @@
     <row r="705">
       <c r="A705" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "profile_id": "0a129ba1-1e8f-490f-8b33-748d6c2db1f3",</t>
+          <t xml:space="preserve">    "profile_id": "dbf32166-b457-4c44-a482-333f013e9541",</t>
         </is>
       </c>
     </row>
@@ -7597,21 +7597,21 @@
     <row r="712">
       <c r="A712" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "entity_id": "26047f96-aba9-4e5f-97eb-a04d18c3e2ce",</t>
+          <t xml:space="preserve">      "entity_id": "c2c5b835-808e-413d-a637-67ece499bbdf",</t>
         </is>
       </c>
     </row>
     <row r="713">
       <c r="A713" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "period_id": "075ce9a3-fc18-4d94-b850-2f7a6e4d0e3f",</t>
+          <t xml:space="preserve">      "period_id": "df6051b0-8cee-4339-8960-bdbb16c31efe",</t>
         </is>
       </c>
     </row>
     <row r="714">
       <c r="A714" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "tenant_id": "3c52af75-856a-4d05-aed4-aa0f5f067823",</t>
+          <t xml:space="preserve">      "tenant_id": "dcba6fad-cdaf-4a38-8bf0-776abb23ecf9",</t>
         </is>
       </c>
     </row>
@@ -7646,7 +7646,7 @@
     <row r="719">
       <c r="A719" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "execution_id": "438cd359-30fc-4896-a3d6-f01396f930d7",</t>
+          <t xml:space="preserve">      "execution_id": "56714a73-6274-4f27-8184-1f903c31ab2e",</t>
         </is>
       </c>
     </row>
@@ -7660,7 +7660,7 @@
     <row r="721">
       <c r="A721" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "engagement_id": "8566cd98-1801-41ee-94c0-604933ca119c",</t>
+          <t xml:space="preserve">      "engagement_id": "4f9da378-404c-4ece-b5f4-6eebb2cb1dff",</t>
         </is>
       </c>
     </row>
@@ -7891,7 +7891,7 @@
     <row r="754">
       <c r="A754" t="inlineStr">
         <is>
-          <t xml:space="preserve">              "da75be6b-463d-44e4-8dc4-1e26094a7ff7"</t>
+          <t xml:space="preserve">              "d6a38fec-06bb-4142-be24-a5abb76c6d31"</t>
         </is>
       </c>
     </row>
@@ -7926,7 +7926,7 @@
     <row r="759">
       <c r="A759" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "rule_record_id": "f387e7fd-fe7a-4fff-893c-f1eb47aa0ed3",</t>
+          <t xml:space="preserve">          "rule_record_id": "4a227430-8782-4779-a651-e7231042a27a",</t>
         </is>
       </c>
     </row>
@@ -8248,7 +8248,7 @@
     <row r="805">
       <c r="A805" t="inlineStr">
         <is>
-          <t xml:space="preserve">              "da75be6b-463d-44e4-8dc4-1e26094a7ff7"</t>
+          <t xml:space="preserve">              "d6a38fec-06bb-4142-be24-a5abb76c6d31"</t>
         </is>
       </c>
     </row>
@@ -8283,7 +8283,7 @@
     <row r="810">
       <c r="A810" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "rule_record_id": "33ed8bae-2f18-4b6a-8347-39373f58e484",</t>
+          <t xml:space="preserve">          "rule_record_id": "8c530841-0422-4d7a-8873-512cc840211e",</t>
         </is>
       </c>
     </row>
@@ -8591,7 +8591,7 @@
     <row r="854">
       <c r="A854" t="inlineStr">
         <is>
-          <t xml:space="preserve">              "da75be6b-463d-44e4-8dc4-1e26094a7ff7"</t>
+          <t xml:space="preserve">              "d6a38fec-06bb-4142-be24-a5abb76c6d31"</t>
         </is>
       </c>
     </row>
@@ -8626,7 +8626,7 @@
     <row r="859">
       <c r="A859" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "rule_record_id": "63b9bd2c-df96-469f-82d3-857205b0f694",</t>
+          <t xml:space="preserve">          "rule_record_id": "35b21af8-1e1c-4fe3-b402-6c26e3f289b4",</t>
         </is>
       </c>
     </row>
@@ -8976,7 +8976,7 @@
     <row r="909">
       <c r="A909" t="inlineStr">
         <is>
-          <t xml:space="preserve">              "da75be6b-463d-44e4-8dc4-1e26094a7ff7"</t>
+          <t xml:space="preserve">              "d6a38fec-06bb-4142-be24-a5abb76c6d31"</t>
         </is>
       </c>
     </row>
@@ -9011,7 +9011,7 @@
     <row r="914">
       <c r="A914" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "rule_record_id": "134ca4a1-d675-4d20-a5cc-25061178240b",</t>
+          <t xml:space="preserve">          "rule_record_id": "3cc2f1e2-0cb1-4fa3-841c-274d6be8fe8b",</t>
         </is>
       </c>
     </row>
@@ -9326,7 +9326,7 @@
     <row r="959">
       <c r="A959" t="inlineStr">
         <is>
-          <t xml:space="preserve">              "da75be6b-463d-44e4-8dc4-1e26094a7ff7"</t>
+          <t xml:space="preserve">              "d6a38fec-06bb-4142-be24-a5abb76c6d31"</t>
         </is>
       </c>
     </row>
@@ -9361,7 +9361,7 @@
     <row r="964">
       <c r="A964" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "rule_record_id": "749bfec7-47a7-4cfb-919f-6c420f9fc15f",</t>
+          <t xml:space="preserve">          "rule_record_id": "7b5603f4-6138-4607-af70-515610f0da73",</t>
         </is>
       </c>
     </row>
@@ -9676,7 +9676,7 @@
     <row r="1009">
       <c r="A1009" t="inlineStr">
         <is>
-          <t xml:space="preserve">              "da75be6b-463d-44e4-8dc4-1e26094a7ff7"</t>
+          <t xml:space="preserve">              "d6a38fec-06bb-4142-be24-a5abb76c6d31"</t>
         </is>
       </c>
     </row>
@@ -9711,7 +9711,7 @@
     <row r="1014">
       <c r="A1014" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "rule_record_id": "a4399843-db68-4b86-8733-f33e5245e9c0",</t>
+          <t xml:space="preserve">          "rule_record_id": "6d9f0a74-5cfe-4f26-b921-cb4c62d57f4b",</t>
         </is>
       </c>
     </row>
@@ -10026,7 +10026,7 @@
     <row r="1059">
       <c r="A1059" t="inlineStr">
         <is>
-          <t xml:space="preserve">              "da75be6b-463d-44e4-8dc4-1e26094a7ff7"</t>
+          <t xml:space="preserve">              "d6a38fec-06bb-4142-be24-a5abb76c6d31"</t>
         </is>
       </c>
     </row>
@@ -10061,7 +10061,7 @@
     <row r="1064">
       <c r="A1064" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "rule_record_id": "599f6bca-5333-467c-bbc9-5b60b04c9b3e",</t>
+          <t xml:space="preserve">          "rule_record_id": "b8285a20-103d-42c9-9cd0-eeadffc93ab1",</t>
         </is>
       </c>
     </row>
@@ -10201,14 +10201,14 @@
     <row r="1084">
       <c r="A1084" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "8816bb6e-d8c5-4b32-aedd-acba6f466682",</t>
+          <t xml:space="preserve">          "id": "fc289c9d-5afa-4467-9efc-5eee990b5b60",</t>
         </is>
       </c>
     </row>
     <row r="1085">
       <c r="A1085" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "sha256": "7ce31010c21c2309ceeee64b6f08535e9fd76e831e50de13686c36437ac5b613",</t>
+          <t xml:space="preserve">          "sha256": "f5242a8d87d47edc13c135a7ddd7ad5e19a561f5c3406f8a175a5341760444b8",</t>
         </is>
       </c>
     </row>
@@ -10271,7 +10271,7 @@
     <row r="1094">
       <c r="A1094" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "5d6b30ea-667e-4f01-8d3b-219507024f74",</t>
+          <t xml:space="preserve">          "id": "7c922cee-c000-47e0-9e18-e1c67f256d14",</t>
         </is>
       </c>
     </row>
@@ -10306,7 +10306,7 @@
     <row r="1099">
       <c r="A1099" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "5151ae5a-ab3c-4239-9116-57444f6179d2",</t>
+          <t xml:space="preserve">          "id": "fdccd6c0-ab9a-4d7c-9480-1cb36f6b8659",</t>
         </is>
       </c>
     </row>
@@ -10341,7 +10341,7 @@
     <row r="1104">
       <c r="A1104" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "07be194f-aefb-4021-891f-f42b00d1d380",</t>
+          <t xml:space="preserve">          "id": "1e5812ed-4402-4b7f-b92c-49b6428c6ec2",</t>
         </is>
       </c>
     </row>
@@ -10376,7 +10376,7 @@
     <row r="1109">
       <c r="A1109" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "26e3325b-a5cb-418e-8025-167c64388709",</t>
+          <t xml:space="preserve">          "id": "3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0",</t>
         </is>
       </c>
     </row>
@@ -10411,7 +10411,7 @@
     <row r="1114">
       <c r="A1114" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "8111fdc0-a0c3-4220-8d4f-506d02e02aed",</t>
+          <t xml:space="preserve">          "id": "2205c942-8a3b-4df5-8539-6470ac261cc8",</t>
         </is>
       </c>
     </row>
@@ -10446,7 +10446,7 @@
     <row r="1119">
       <c r="A1119" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "c5f2f746-f2ee-44cb-987c-56136d5c2de1",</t>
+          <t xml:space="preserve">          "id": "b243bb9b-6bbb-4c0c-bd5b-5d1c04d48f06",</t>
         </is>
       </c>
     </row>
@@ -10481,7 +10481,7 @@
     <row r="1124">
       <c r="A1124" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "b7bc0e8e-c44c-4000-bc9b-6575a6a3f090",</t>
+          <t xml:space="preserve">          "id": "fb515fbf-b17a-4def-9671-dd74a6b9e094",</t>
         </is>
       </c>
     </row>
@@ -10516,7 +10516,7 @@
     <row r="1129">
       <c r="A1129" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "bec5f73f-4547-4fa6-b494-4636bbb1ae62",</t>
+          <t xml:space="preserve">          "id": "6f8b9d96-c0ae-436b-85c0-339a0c4aa4d9",</t>
         </is>
       </c>
     </row>
@@ -10551,7 +10551,7 @@
     <row r="1134">
       <c r="A1134" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "3bcba9a4-298d-403c-bd92-b88dcd0de1e6",</t>
+          <t xml:space="preserve">          "id": "fa126d00-0e5e-42e4-b043-4938f4c66cd9",</t>
         </is>
       </c>
     </row>
@@ -10586,7 +10586,7 @@
     <row r="1139">
       <c r="A1139" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "eaf1cd80-da44-4287-9129-98e9e720b8a0",</t>
+          <t xml:space="preserve">          "id": "51c8f8a1-5c9a-4d37-8453-a21c548c739d",</t>
         </is>
       </c>
     </row>
@@ -10621,7 +10621,7 @@
     <row r="1144">
       <c r="A1144" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "6a96a1eb-21dd-4cd6-b52d-39e1d24c5c8b",</t>
+          <t xml:space="preserve">          "id": "f17b2344-beab-4a85-ac9c-2316b5015994",</t>
         </is>
       </c>
     </row>
@@ -10656,7 +10656,7 @@
     <row r="1149">
       <c r="A1149" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "0a129ba1-1e8f-490f-8b33-748d6c2db1f3",</t>
+          <t xml:space="preserve">          "id": "dbf32166-b457-4c44-a482-333f013e9541",</t>
         </is>
       </c>
     </row>
@@ -10705,7 +10705,7 @@
     <row r="1156">
       <c r="A1156" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "f387e7fd-fe7a-4fff-893c-f1eb47aa0ed3",</t>
+          <t xml:space="preserve">          "id": "4a227430-8782-4779-a651-e7231042a27a",</t>
         </is>
       </c>
     </row>
@@ -10754,7 +10754,7 @@
     <row r="1163">
       <c r="A1163" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "33ed8bae-2f18-4b6a-8347-39373f58e484",</t>
+          <t xml:space="preserve">          "id": "8c530841-0422-4d7a-8873-512cc840211e",</t>
         </is>
       </c>
     </row>
@@ -10803,7 +10803,7 @@
     <row r="1170">
       <c r="A1170" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "63b9bd2c-df96-469f-82d3-857205b0f694",</t>
+          <t xml:space="preserve">          "id": "35b21af8-1e1c-4fe3-b402-6c26e3f289b4",</t>
         </is>
       </c>
     </row>
@@ -10852,7 +10852,7 @@
     <row r="1177">
       <c r="A1177" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "134ca4a1-d675-4d20-a5cc-25061178240b",</t>
+          <t xml:space="preserve">          "id": "3cc2f1e2-0cb1-4fa3-841c-274d6be8fe8b",</t>
         </is>
       </c>
     </row>
@@ -10901,7 +10901,7 @@
     <row r="1184">
       <c r="A1184" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "749bfec7-47a7-4cfb-919f-6c420f9fc15f",</t>
+          <t xml:space="preserve">          "id": "7b5603f4-6138-4607-af70-515610f0da73",</t>
         </is>
       </c>
     </row>
@@ -10950,7 +10950,7 @@
     <row r="1191">
       <c r="A1191" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "a4399843-db68-4b86-8733-f33e5245e9c0",</t>
+          <t xml:space="preserve">          "id": "6d9f0a74-5cfe-4f26-b921-cb4c62d57f4b",</t>
         </is>
       </c>
     </row>
@@ -10999,7 +10999,7 @@
     <row r="1198">
       <c r="A1198" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "599f6bca-5333-467c-bbc9-5b60b04c9b3e",</t>
+          <t xml:space="preserve">          "id": "b8285a20-103d-42c9-9cd0-eeadffc93ab1",</t>
         </is>
       </c>
     </row>
@@ -11048,7 +11048,7 @@
     <row r="1205">
       <c r="A1205" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "d56ca2f7-3b45-4fc5-87b1-a298cb1f4645",</t>
+          <t xml:space="preserve">          "id": "b39363ca-4043-4e47-924e-d492e6537e59",</t>
         </is>
       </c>
     </row>
@@ -11097,14 +11097,14 @@
     <row r="1212">
       <c r="A1212" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "26e3325b-a5cb-418e-8025-167c64388709",</t>
+          <t xml:space="preserve">          "id": "30e11100-a98b-4418-806b-7b0062760904",</t>
         </is>
       </c>
     </row>
     <row r="1213">
       <c r="A1213" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "kind": "ifrs-note",</t>
+          <t xml:space="preserve">          "kind": "tp-far",</t>
         </is>
       </c>
     </row>
@@ -11146,7 +11146,7 @@
     <row r="1219">
       <c r="A1219" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "98678ad6-7d06-424d-ac6a-0c1f973f72ed",</t>
+          <t xml:space="preserve">          "id": "8f8e7a1e-a7bc-4812-91f0-d76c99dcf630",</t>
         </is>
       </c>
     </row>
@@ -11195,14 +11195,14 @@
     <row r="1226">
       <c r="A1226" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "e94f2c1e-966f-4abb-87a5-66d8467d8f35",</t>
+          <t xml:space="preserve">          "id": "3e14c2cf-ab13-4b8c-9cad-bb5430e0fce0",</t>
         </is>
       </c>
     </row>
     <row r="1227">
       <c r="A1227" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "kind": "tp-far",</t>
+          <t xml:space="preserve">          "kind": "ifrs-note",</t>
         </is>
       </c>
     </row>
@@ -11244,7 +11244,7 @@
     <row r="1233">
       <c r="A1233" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "ad4c54ff-da6c-4474-a0d7-99c82e42ba9b",</t>
+          <t xml:space="preserve">          "id": "78c8e4a2-30a6-4043-ab30-8f30b5206b63",</t>
         </is>
       </c>
     </row>
@@ -11293,7 +11293,7 @@
     <row r="1240">
       <c r="A1240" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "249b5cc3-1aa2-4fc2-a638-fa4a21f8b192",</t>
+          <t xml:space="preserve">          "id": "1fdbf156-cf26-4343-ae8e-35306c4317d4",</t>
         </is>
       </c>
     </row>
@@ -11342,7 +11342,7 @@
     <row r="1247">
       <c r="A1247" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "0ceeb1f1-b2a2-43ec-8d87-840f74b2dd70",</t>
+          <t xml:space="preserve">          "id": "4942fe08-8c8c-47a8-8d93-b25684055404",</t>
         </is>
       </c>
     </row>
@@ -11391,7 +11391,7 @@
     <row r="1254">
       <c r="A1254" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "60346b5b-473b-4889-a5da-68b017ca186b",</t>
+          <t xml:space="preserve">          "id": "be3f8a86-2ec4-4216-a9d5-aad320edb4a7",</t>
         </is>
       </c>
     </row>
@@ -11440,7 +11440,7 @@
     <row r="1261">
       <c r="A1261" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "8534d3b8-8b3a-44de-b207-57cc951802f9",</t>
+          <t xml:space="preserve">          "id": "3cc9dc57-ce14-47b2-afe4-053e2ddf3ce3",</t>
         </is>
       </c>
     </row>
@@ -11489,7 +11489,7 @@
     <row r="1268">
       <c r="A1268" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "749bfec7-47a7-4cfb-919f-6c420f9fc15f",</t>
+          <t xml:space="preserve">          "id": "7b5603f4-6138-4607-af70-515610f0da73",</t>
         </is>
       </c>
     </row>
@@ -11538,7 +11538,7 @@
     <row r="1275">
       <c r="A1275" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "4728be13-cd4e-4cff-b944-aaa72314e339",</t>
+          <t xml:space="preserve">          "id": "a068f299-a348-4b3c-bdd6-72eddf9ad9c2",</t>
         </is>
       </c>
     </row>
@@ -11552,7 +11552,7 @@
     <row r="1277">
       <c r="A1277" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "sha256": "bb6f6c59ca6fe7f3b2a629ba29c663b12a97df4414d9aad8e355a7a861a82292"</t>
+          <t xml:space="preserve">          "sha256": "bf71045089aa949cc8b15a40099a37437bd3959c1aabfcf02d7ab34f63fc6b76"</t>
         </is>
       </c>
     </row>
@@ -11573,7 +11573,7 @@
     <row r="1280">
       <c r="A1280" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "3ad8dcc4-73bb-4757-860b-d47162b2a4cf",</t>
+          <t xml:space="preserve">          "id": "3e0e7d7b-c078-41f1-887b-adbd588c0d57",</t>
         </is>
       </c>
     </row>
@@ -11587,7 +11587,7 @@
     <row r="1282">
       <c r="A1282" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "sha256": "938fe13b721d15eebe42e4915709301cad961dd4f53e781a1f34575768e4a668"</t>
+          <t xml:space="preserve">          "sha256": "d6cb1126efd9719296f6f085bf132532baa9572aeb6618772d51dc7d65e6e228"</t>
         </is>
       </c>
     </row>
@@ -11608,7 +11608,7 @@
     <row r="1285">
       <c r="A1285" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "8a856c62-8985-46d5-913a-50057385d3f4",</t>
+          <t xml:space="preserve">          "id": "4852218e-f3f3-4ac7-93dc-f5a525cf96c5",</t>
         </is>
       </c>
     </row>
@@ -11622,7 +11622,7 @@
     <row r="1287">
       <c r="A1287" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "sha256": "11a5e9130b9b012d21bd7ed155d7173f79fb0221274b4c0d06f2ac557133d3bf"</t>
+          <t xml:space="preserve">          "sha256": "384d550fadd1c9918ea31b0df66c48fd83576321952e40c92268e587b5166633"</t>
         </is>
       </c>
     </row>
@@ -11706,7 +11706,7 @@
     <row r="1299">
       <c r="A1299" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "71f987c2-5e78-4792-85c8-a0f350bb8c1b",</t>
+          <t xml:space="preserve">          "id": "0bb595aa-ad4f-4bd1-a3a3-85318c18eb71",</t>
         </is>
       </c>
     </row>
@@ -11776,7 +11776,7 @@
     <row r="1309">
       <c r="A1309" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "7976f107-0938-4998-be7b-8b97662b9b33",</t>
+          <t xml:space="preserve">          "id": "0cac4b13-42bd-4775-8180-ea5771bb4fec",</t>
         </is>
       </c>
     </row>
@@ -11846,7 +11846,7 @@
     <row r="1319">
       <c r="A1319" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "92ab2c14-847d-4b5b-8870-63f745d300cc",</t>
+          <t xml:space="preserve">          "id": "81c193a5-b3d2-4819-82ec-eb7293dba45d",</t>
         </is>
       </c>
     </row>
@@ -11916,7 +11916,7 @@
     <row r="1329">
       <c r="A1329" t="inlineStr">
         <is>
-          <t xml:space="preserve">          "id": "a754e03d-faaa-434a-a71c-5d745946bda9",</t>
+          <t xml:space="preserve">          "id": "9325fbd0-d504-432a-b857-33c859d800bb",</t>
         </is>
       </c>
     </row>
@@ -12007,7 +12007,7 @@
     <row r="1342">
       <c r="A1342" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "profile_id": "0a129ba1-1e8f-490f-8b33-748d6c2db1f3",</t>
+          <t xml:space="preserve">        "profile_id": "dbf32166-b457-4c44-a482-333f013e9541",</t>
         </is>
       </c>
     </row>
@@ -12063,7 +12063,7 @@
     <row r="1350">
       <c r="A1350" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "financial_source_id": "cf928a21-d968-43bd-af21-cbe63c33f5f4",</t>
+          <t xml:space="preserve">    "financial_source_id": "0dc3d575-c9b9-4d71-bb27-b2b7bd223373",</t>
         </is>
       </c>
     </row>
@@ -12091,7 +12091,7 @@
     <row r="1354">
       <c r="A1354" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "run_id": "4728be13-cd4e-4cff-b944-aaa72314e339",</t>
+          <t xml:space="preserve">        "run_id": "3e0e7d7b-c078-41f1-887b-adbd588c0d57",</t>
         </is>
       </c>
     </row>
@@ -12147,7 +12147,7 @@
     <row r="1362">
       <c r="A1362" t="inlineStr">
         <is>
-          <t xml:space="preserve">        "run_id": "8a856c62-8985-46d5-913a-50057385d3f4",</t>
+          <t xml:space="preserve">        "run_id": "4852218e-f3f3-4ac7-93dc-f5a525cf96c5",</t>
         </is>
       </c>
     </row>
@@ -12266,7 +12266,7 @@
     <row r="1379">
       <c r="A1379" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "financial_reconciliation_run_id": "3ad8dcc4-73bb-4757-860b-d47162b2a4cf"</t>
+          <t xml:space="preserve">    "financial_reconciliation_run_id": "a068f299-a348-4b3c-bdd6-72eddf9ad9c2"</t>
         </is>
       </c>
     </row>

</xml_diff>